<commit_message>
chore(jdt): remplissage du jdt pour le 11.09.2026
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE370EEF-CF31-4089-9C5F-99150B5B2C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB389CB3-CD28-420B-8B72-93A61C057DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="49">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -166,7 +166,37 @@
     <t>Doc</t>
   </si>
   <si>
-    <t>Je finis la documentation nécessaire é la release (rendu).</t>
+    <t>Je finis la documentation nécessaire à la release (rendu).</t>
+  </si>
+  <si>
+    <t>Je finis les user stories (modifications possibles dans le futur).</t>
+  </si>
+  <si>
+    <t>https://github.com/users/yohannf-222/projects/1</t>
+  </si>
+  <si>
+    <t>Cdc</t>
+  </si>
+  <si>
+    <t>Je repasse rapidement sur le cdc pour me mettre sur la voie du travail.</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>https://apps.pm2etml.ch/jobDefinitions/99</t>
+  </si>
+  <si>
+    <t>Je télécharge la base sur pm2etml et essaye de me situer dedans avec mon idée de projet.</t>
+  </si>
+  <si>
+    <t>Compte rendu de la release v1</t>
+  </si>
+  <si>
+    <t>Je modifie mes US suite aux commentaires du Cdp.</t>
+  </si>
+  <si>
+    <t>Le Cdp commente ma release v1 et me dis ce qui est à revoir.</t>
   </si>
 </sst>
 </file>
@@ -412,7 +442,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -550,6 +580,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1084,41 +1118,77 @@
       <c r="E15" s="35"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="28"/>
+      <c r="A16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46276</v>
+      </c>
+      <c r="C16" s="5">
+        <v>80</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
+      <c r="A17" s="7" t="s">
+        <v>41</v>
+      </c>
       <c r="B17" s="36"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
+      <c r="C17" s="8">
+        <v>10</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
+      <c r="A18" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="B18" s="36"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="8"/>
-    </row>
-    <row r="19" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
+      <c r="C18" s="8">
+        <v>45</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="42" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>46</v>
+      </c>
       <c r="B19" s="36"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
+      <c r="C19" s="8">
+        <v>25</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>48</v>
+      </c>
       <c r="E19" s="8"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
+      <c r="A20" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="B20" s="37"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
+      <c r="C20" s="10">
+        <v>20</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>47</v>
+      </c>
       <c r="E20" s="10"/>
     </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
@@ -2088,7 +2158,7 @@
       <c r="B153" s="27"/>
       <c r="C153" s="15">
         <f>MROUND(SUM(C6:C152) /60,0.2)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D153" s="16"/>
       <c r="E153" s="17"/>
@@ -2165,59 +2235,47 @@
   <hyperlinks>
     <hyperlink ref="E6" r:id="rId1" display="https://github.com/yohannf-222/Projet-320-ShootMeUp-YFS" xr:uid="{4F6F040C-0604-4D50-B72F-88A593B382CF}"/>
     <hyperlink ref="E14" r:id="rId2" display="https://github.com/users/yohannf-222/projects/1" xr:uid="{2674A8DD-7527-4DBA-B059-08BA3C423966}"/>
+    <hyperlink ref="E18" r:id="rId3" xr:uid="{CA435077-98B4-4033-B7A1-B11620AF26C6}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
   </headerFooter>
-  <legacyDrawingHF r:id="rId4"/>
+  <legacyDrawingHF r:id="rId5"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="4356f79f-5386-4bda-9d92-82d8bd7b074e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3eb094ff-ec8d-44d8-be06-94ad3ec8832a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010051C931FEC57CD24D841BB655C8BA0DFF" ma:contentTypeVersion="11" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="b1e7b700e38e961fcf6b815c67f211ba">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" xmlns:ns3="4356f79f-5386-4bda-9d92-82d8bd7b074e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="90ca33f58fbebba084d82664f7828ed0" ns2:_="" ns3:_="">
-    <xsd:import namespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
-    <xsd:import namespace="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
+    <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element name="documentManagement">
             <xsd:complexType>
               <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaLengthInSeconds" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -2225,72 +2283,60 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3eb094ff-ec8d-44d8-be06-94ad3ec8832a" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="8" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+    <xsd:element name="MediaServiceFastMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="11" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+    <xsd:element name="_activity" ma:index="12" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="5cfe7824-1d92-4d19-9a43-1c93e0eb464f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
+    <xsd:element name="MediaServiceSystemTags" ma:index="13" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="18" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+    <xsd:element name="MediaLengthInSeconds" ma:index="17" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
+        <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4356f79f-5386-4bda-9d92-82d8bd7b074e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{4ed9f543-e2bd-4fe6-b9a6-97a4976c5506}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4356f79f-5386-4bda-9d92-82d8bd7b074e">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -2392,40 +2438,39 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14CC8145-5BC5-4FF1-BE7C-3D8C788DCF73}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="3eb094ff-ec8d-44d8-be06-94ad3ec8832a"/>
-    <ds:schemaRef ds:uri="4356f79f-5386-4bda-9d92-82d8bd7b074e"/>
+    <ds:schemaRef ds:uri="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -2434,4 +2479,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(Projet): Adapter le projet à la base fournie
je n'utilisais malencontreusement pas la base fournie par erreur.
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB389CB3-CD28-420B-8B72-93A61C057DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E26DA5E-83BC-4FF7-B824-BA89FFC5BE7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$153</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$39</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -198,12 +198,18 @@
   <si>
     <t>Le Cdp commente ma release v1 et me dis ce qui est à revoir.</t>
   </si>
+  <si>
+    <t>Début Projet</t>
+  </si>
+  <si>
+    <t>J'essaye de implémenter un joueur (classe, instanciation, image).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Century Gothic"/>
@@ -253,12 +259,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Century Gothic"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -442,7 +442,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -525,7 +525,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -533,34 +532,26 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -569,20 +560,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -901,7 +888,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -918,10 +905,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="38"/>
+      <c r="C1" s="29"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -933,10 +920,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="38"/>
+      <c r="C2" s="29"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -948,10 +935,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="38"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -963,12 +950,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -991,7 +978,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="30">
+      <c r="B6" s="33">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1008,7 +995,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="36"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1021,7 +1008,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="36"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1034,16 +1021,19 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35"/>
+      <c r="B9" s="36">
+        <f>SUM(C10:C14)</f>
+        <v>180</v>
+      </c>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="38"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="30">
+      <c r="B10" s="33">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1052,13 +1042,13 @@
       <c r="D10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="28"/>
+      <c r="E10" s="27"/>
     </row>
     <row r="11" spans="1:5" s="23" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="36"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1071,7 +1061,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="36"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1084,7 +1074,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="36"/>
+      <c r="B13" s="34"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1097,7 +1087,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="37"/>
+      <c r="B14" s="35"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1112,16 +1102,19 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="33"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
+      <c r="B15" s="36">
+        <f>SUM(C16:C20)</f>
+        <v>180</v>
+      </c>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="38"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="33">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1130,7 +1123,7 @@
       <c r="D16" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="E16" s="27" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1138,7 +1131,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="36"/>
+      <c r="B17" s="34"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1151,14 +1144,14 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="36"/>
+      <c r="B18" s="34"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="42" t="s">
+      <c r="E18" s="28" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1166,7 +1159,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="36"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1179,7 +1172,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="37"/>
+      <c r="B20" s="35"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1192,42 +1185,53 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="33"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="35"/>
+      <c r="B21" s="36">
+        <f>SUM(C22:C26)</f>
+        <v>60</v>
+      </c>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="38"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="28"/>
+      <c r="A22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="33">
+        <v>46283</v>
+      </c>
+      <c r="C22" s="5">
+        <v>60</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" s="27"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="36"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="8"/>
       <c r="D23" s="9"/>
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
-      <c r="B24" s="36"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="8"/>
       <c r="D24" s="9"/>
       <c r="E24" s="8"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="36"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="37"/>
+      <c r="B26" s="35"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1236,946 +1240,120 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="35"/>
+      <c r="B27" s="36">
+        <f>SUM(C28:C32)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="38"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
-      <c r="B28" s="30"/>
+      <c r="B28" s="33"/>
       <c r="C28" s="13"/>
       <c r="D28" s="14"/>
-      <c r="E28" s="28"/>
+      <c r="E28" s="27"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
-      <c r="B29" s="36"/>
+      <c r="B29" s="34"/>
       <c r="C29" s="8"/>
       <c r="D29" s="9"/>
-      <c r="E29" s="28"/>
+      <c r="E29" s="27"/>
     </row>
     <row r="30" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
-      <c r="B30" s="36"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
-      <c r="E30" s="28"/>
+      <c r="E30" s="27"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="36"/>
+      <c r="B31" s="34"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="37"/>
+      <c r="B32" s="35"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
-    <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="33"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="35"/>
+      <c r="B33" s="36">
+        <f>SUM(C34:C38)</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="38"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="30"/>
+      <c r="B34" s="33"/>
       <c r="C34" s="5"/>
       <c r="D34" s="6"/>
-      <c r="E34" s="28"/>
+      <c r="E34" s="27"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="36"/>
+      <c r="B35" s="34"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
-      <c r="E35" s="28"/>
+      <c r="E35" s="27"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="36"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
-      <c r="E36" s="28"/>
+      <c r="E36" s="27"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="36"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="37"/>
+      <c r="B38" s="35"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
     </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B39" s="33"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="35"/>
-    </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="4"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="25"/>
-      <c r="E40" s="5"/>
-    </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="7"/>
-      <c r="B41" s="36"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="28"/>
-    </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7"/>
-      <c r="B42" s="36"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="28"/>
-    </row>
-    <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="7"/>
-      <c r="B43" s="36"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="8"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="10"/>
-      <c r="B44" s="37"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="10"/>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="12"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="34"/>
-      <c r="E45" s="35"/>
-    </row>
-    <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="4"/>
-      <c r="B46" s="30"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="28"/>
-    </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="7"/>
-      <c r="B47" s="36"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="28"/>
-    </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7"/>
-      <c r="B48" s="36"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="8"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="7"/>
-      <c r="B49" s="36"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="8"/>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="10"/>
-      <c r="B50" s="37"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="10"/>
-    </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B51" s="33"/>
-      <c r="C51" s="34"/>
-      <c r="D51" s="34"/>
-      <c r="E51" s="35"/>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="4"/>
-      <c r="B52" s="30"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="28"/>
-    </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="36"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="28"/>
-    </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="7"/>
-      <c r="B54" s="36"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="8"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="7"/>
-      <c r="B55" s="36"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="8"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10"/>
-      <c r="B56" s="37"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="10"/>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B57" s="33"/>
-      <c r="C57" s="34"/>
-      <c r="D57" s="34"/>
-      <c r="E57" s="35"/>
-    </row>
-    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="13"/>
-      <c r="B58" s="30"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="28"/>
-    </row>
-    <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="8"/>
-      <c r="B59" s="36"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="28"/>
-    </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="8"/>
-      <c r="B60" s="36"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="8"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="8"/>
-      <c r="B61" s="36"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="8"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="8"/>
-      <c r="B62" s="37"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B63" s="33"/>
-      <c r="C63" s="34"/>
-      <c r="D63" s="34"/>
-      <c r="E63" s="35"/>
-    </row>
-    <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="8"/>
-      <c r="B64" s="30"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="28"/>
-    </row>
-    <row r="65" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="36"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="8"/>
-      <c r="B66" s="36"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="8"/>
-    </row>
-    <row r="67" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="8"/>
-      <c r="B67" s="36"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="8"/>
-      <c r="B68" s="37"/>
-      <c r="E68" s="8"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B69" s="33"/>
-      <c r="C69" s="34"/>
-      <c r="D69" s="34"/>
-      <c r="E69" s="35"/>
-    </row>
-    <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="8"/>
-      <c r="B70" s="30"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="28"/>
-    </row>
-    <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="8"/>
-      <c r="B71" s="36"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="8"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="8"/>
-      <c r="B72" s="36"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="8"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="8"/>
-      <c r="B73" s="36"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="8"/>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="8"/>
-      <c r="B74" s="37"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="9"/>
-      <c r="E74" s="8"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B75" s="33"/>
-      <c r="C75" s="34"/>
-      <c r="D75" s="34"/>
-      <c r="E75" s="35"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="13"/>
-      <c r="B76" s="30"/>
-      <c r="C76" s="13"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="28"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="8"/>
-      <c r="B77" s="36"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="8"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="8"/>
-      <c r="B78" s="36"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="29"/>
-      <c r="E78" s="8"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="8"/>
-      <c r="B79" s="36"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="8"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="8"/>
-      <c r="B80" s="37"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="9"/>
-      <c r="E80" s="8"/>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B81" s="33"/>
-      <c r="C81" s="34"/>
-      <c r="D81" s="34"/>
-      <c r="E81" s="35"/>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="13"/>
-      <c r="B82" s="30"/>
-      <c r="C82" s="13"/>
-      <c r="D82" s="14"/>
-      <c r="E82" s="28"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="13"/>
-      <c r="B83" s="31"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="14"/>
-      <c r="E83" s="28"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="8"/>
-      <c r="B84" s="31"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="9"/>
-      <c r="E84" s="8"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="8"/>
-      <c r="B85" s="31"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="9"/>
-      <c r="E85" s="8"/>
-    </row>
-    <row r="86" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="8"/>
-      <c r="B86" s="32"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="9"/>
-      <c r="E86" s="8"/>
-    </row>
-    <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B87" s="33"/>
-      <c r="C87" s="34"/>
-      <c r="D87" s="34"/>
-      <c r="E87" s="35"/>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="13"/>
-      <c r="B88" s="30"/>
-      <c r="C88" s="13"/>
-      <c r="D88" s="14"/>
-      <c r="E88" s="28"/>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="13"/>
-      <c r="B89" s="31"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="14"/>
-      <c r="E89" s="28"/>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="8"/>
-      <c r="B90" s="31"/>
-      <c r="C90" s="8"/>
-      <c r="D90" s="9"/>
-      <c r="E90" s="8"/>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="8"/>
-      <c r="B91" s="31"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="9"/>
-      <c r="E91" s="8"/>
-    </row>
-    <row r="92" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="8"/>
-      <c r="B92" s="32"/>
-      <c r="C92" s="8"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="8"/>
-    </row>
-    <row r="93" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B93" s="33"/>
-      <c r="C93" s="34"/>
-      <c r="D93" s="34"/>
-      <c r="E93" s="35"/>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="13"/>
-      <c r="B94" s="30"/>
-      <c r="C94" s="13"/>
-      <c r="D94" s="14"/>
-      <c r="E94" s="28"/>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="13"/>
-      <c r="B95" s="31"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="14"/>
-      <c r="E95" s="28"/>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="8"/>
-      <c r="B96" s="31"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="9"/>
-      <c r="E96" s="8"/>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="8"/>
-      <c r="B97" s="31"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="9"/>
-      <c r="E97" s="8"/>
-    </row>
-    <row r="98" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="8"/>
-      <c r="B98" s="32"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="9"/>
-      <c r="E98" s="8"/>
-    </row>
-    <row r="99" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B99" s="33"/>
-      <c r="C99" s="34"/>
-      <c r="D99" s="34"/>
-      <c r="E99" s="35"/>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="13"/>
-      <c r="B100" s="30"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="14"/>
-      <c r="E100" s="28"/>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="13"/>
-      <c r="B101" s="31"/>
-      <c r="C101" s="8"/>
-      <c r="D101" s="14"/>
-      <c r="E101" s="28"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="8"/>
-      <c r="B102" s="31"/>
-      <c r="C102" s="8"/>
-      <c r="D102" s="9"/>
-      <c r="E102" s="8"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="8"/>
-      <c r="B103" s="31"/>
-      <c r="C103" s="8"/>
-      <c r="D103" s="9"/>
-      <c r="E103" s="8"/>
-    </row>
-    <row r="104" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="8"/>
-      <c r="B104" s="32"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="9"/>
-      <c r="E104" s="8"/>
-    </row>
-    <row r="105" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B105" s="33"/>
-      <c r="C105" s="34"/>
-      <c r="D105" s="34"/>
-      <c r="E105" s="35"/>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="13"/>
-      <c r="B106" s="30"/>
-      <c r="C106" s="13"/>
-      <c r="D106" s="14"/>
-      <c r="E106" s="28"/>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="13"/>
-      <c r="B107" s="31"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="14"/>
-      <c r="E107" s="28"/>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="8"/>
-      <c r="B108" s="31"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="9"/>
-      <c r="E108" s="8"/>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="8"/>
-      <c r="B109" s="31"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="9"/>
-      <c r="E109" s="8"/>
-    </row>
-    <row r="110" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="8"/>
-      <c r="B110" s="32"/>
-      <c r="C110" s="8"/>
-      <c r="D110" s="9"/>
-      <c r="E110" s="8"/>
-    </row>
-    <row r="111" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B111" s="33"/>
-      <c r="C111" s="34"/>
-      <c r="D111" s="34"/>
-      <c r="E111" s="35"/>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="13"/>
-      <c r="B112" s="30"/>
-      <c r="C112" s="13"/>
-      <c r="D112" s="14"/>
-      <c r="E112" s="28"/>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="13"/>
-      <c r="B113" s="31"/>
-      <c r="C113" s="8"/>
-      <c r="D113" s="14"/>
-      <c r="E113" s="28"/>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="8"/>
-      <c r="B114" s="31"/>
-      <c r="C114" s="8"/>
-      <c r="D114" s="9"/>
-      <c r="E114" s="8"/>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="8"/>
-      <c r="B115" s="31"/>
-      <c r="C115" s="8"/>
-      <c r="D115" s="9"/>
-      <c r="E115" s="8"/>
-    </row>
-    <row r="116" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="8"/>
-      <c r="B116" s="32"/>
-      <c r="C116" s="8"/>
-      <c r="D116" s="9"/>
-      <c r="E116" s="8"/>
-    </row>
-    <row r="117" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B117" s="33"/>
-      <c r="C117" s="34"/>
-      <c r="D117" s="34"/>
-      <c r="E117" s="35"/>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" s="13"/>
-      <c r="B118" s="30"/>
-      <c r="C118" s="13"/>
-      <c r="D118" s="14"/>
-      <c r="E118" s="28"/>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="13"/>
-      <c r="B119" s="31"/>
-      <c r="C119" s="8"/>
-      <c r="D119" s="14"/>
-      <c r="E119" s="28"/>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="8"/>
-      <c r="B120" s="31"/>
-      <c r="C120" s="8"/>
-      <c r="D120" s="9"/>
-      <c r="E120" s="8"/>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="8"/>
-      <c r="B121" s="31"/>
-      <c r="C121" s="8"/>
-      <c r="D121" s="9"/>
-      <c r="E121" s="8"/>
-    </row>
-    <row r="122" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="8"/>
-      <c r="B122" s="32"/>
-      <c r="C122" s="8"/>
-      <c r="D122" s="9"/>
-      <c r="E122" s="8"/>
-    </row>
-    <row r="123" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B123" s="33"/>
-      <c r="C123" s="34"/>
-      <c r="D123" s="34"/>
-      <c r="E123" s="35"/>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="13"/>
-      <c r="B124" s="30"/>
-      <c r="C124" s="13"/>
-      <c r="D124" s="14"/>
-      <c r="E124" s="28"/>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="13"/>
-      <c r="B125" s="31"/>
-      <c r="C125" s="8"/>
-      <c r="D125" s="14"/>
-      <c r="E125" s="28"/>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" s="8"/>
-      <c r="B126" s="31"/>
-      <c r="C126" s="8"/>
-      <c r="D126" s="9"/>
-      <c r="E126" s="8"/>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" s="8"/>
-      <c r="B127" s="31"/>
-      <c r="C127" s="8"/>
-      <c r="D127" s="9"/>
-      <c r="E127" s="8"/>
-    </row>
-    <row r="128" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="8"/>
-      <c r="B128" s="32"/>
-      <c r="C128" s="8"/>
-      <c r="D128" s="9"/>
-      <c r="E128" s="8"/>
-    </row>
-    <row r="129" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B129" s="33"/>
-      <c r="C129" s="34"/>
-      <c r="D129" s="34"/>
-      <c r="E129" s="35"/>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" s="13"/>
-      <c r="B130" s="30"/>
-      <c r="C130" s="13"/>
-      <c r="D130" s="14"/>
-      <c r="E130" s="28"/>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A131" s="13"/>
-      <c r="B131" s="31"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="14"/>
-      <c r="E131" s="28"/>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" s="8"/>
-      <c r="B132" s="31"/>
-      <c r="C132" s="8"/>
-      <c r="D132" s="9"/>
-      <c r="E132" s="8"/>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="8"/>
-      <c r="B133" s="31"/>
-      <c r="C133" s="8"/>
-      <c r="D133" s="9"/>
-      <c r="E133" s="8"/>
-    </row>
-    <row r="134" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="8"/>
-      <c r="B134" s="32"/>
-      <c r="C134" s="8"/>
-      <c r="D134" s="9"/>
-      <c r="E134" s="8"/>
-    </row>
-    <row r="135" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B135" s="33"/>
-      <c r="C135" s="34"/>
-      <c r="D135" s="34"/>
-      <c r="E135" s="35"/>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" s="13"/>
-      <c r="B136" s="30"/>
-      <c r="C136" s="13"/>
-      <c r="D136" s="14"/>
-      <c r="E136" s="28"/>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" s="13"/>
-      <c r="B137" s="31"/>
-      <c r="C137" s="8"/>
-      <c r="D137" s="14"/>
-      <c r="E137" s="28"/>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="8"/>
-      <c r="B138" s="31"/>
-      <c r="C138" s="8"/>
-      <c r="D138" s="9"/>
-      <c r="E138" s="8"/>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" s="8"/>
-      <c r="B139" s="31"/>
-      <c r="C139" s="8"/>
-      <c r="D139" s="9"/>
-      <c r="E139" s="8"/>
-    </row>
-    <row r="140" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="8"/>
-      <c r="B140" s="32"/>
-      <c r="C140" s="8"/>
-      <c r="D140" s="9"/>
-      <c r="E140" s="8"/>
-    </row>
-    <row r="141" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B141" s="33"/>
-      <c r="C141" s="34"/>
-      <c r="D141" s="34"/>
-      <c r="E141" s="35"/>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A142" s="13"/>
-      <c r="B142" s="30"/>
-      <c r="C142" s="13"/>
-      <c r="D142" s="14"/>
-      <c r="E142" s="28"/>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A143" s="13"/>
-      <c r="B143" s="31"/>
-      <c r="C143" s="8"/>
-      <c r="D143" s="14"/>
-      <c r="E143" s="28"/>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A144" s="8"/>
-      <c r="B144" s="31"/>
-      <c r="C144" s="8"/>
-      <c r="D144" s="9"/>
-      <c r="E144" s="8"/>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A145" s="8"/>
-      <c r="B145" s="31"/>
-      <c r="C145" s="8"/>
-      <c r="D145" s="9"/>
-      <c r="E145" s="8"/>
-    </row>
-    <row r="146" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="8"/>
-      <c r="B146" s="32"/>
-      <c r="C146" s="8"/>
-      <c r="D146" s="9"/>
-      <c r="E146" s="8"/>
-    </row>
-    <row r="147" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B147" s="33"/>
-      <c r="C147" s="34"/>
-      <c r="D147" s="34"/>
-      <c r="E147" s="35"/>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A148" s="13"/>
-      <c r="B148" s="30"/>
-      <c r="C148" s="13"/>
-      <c r="D148" s="14"/>
-      <c r="E148" s="28"/>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A149" s="13"/>
-      <c r="B149" s="31"/>
-      <c r="C149" s="8"/>
-      <c r="D149" s="14"/>
-      <c r="E149" s="28"/>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" s="8"/>
-      <c r="B150" s="31"/>
-      <c r="C150" s="8"/>
-      <c r="D150" s="9"/>
-      <c r="E150" s="8"/>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A151" s="8"/>
-      <c r="B151" s="31"/>
-      <c r="C151" s="8"/>
-      <c r="D151" s="9"/>
-      <c r="E151" s="8"/>
-    </row>
-    <row r="152" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A152" s="8"/>
-      <c r="B152" s="32"/>
-      <c r="C152" s="8"/>
-      <c r="D152" s="9"/>
-      <c r="E152" s="8"/>
-    </row>
-    <row r="153" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="26" t="s">
+    <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B153" s="27"/>
-      <c r="C153" s="15">
-        <f>MROUND(SUM(C6:C152) /60,0.2)</f>
-        <v>9</v>
-      </c>
-      <c r="D153" s="16"/>
-      <c r="E153" s="17"/>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A155" s="18" t="s">
+      <c r="B39" s="26"/>
+      <c r="C39" s="15">
+        <f>MROUND(SUM(C6:C38) /60,0.2)</f>
+        <v>10</v>
+      </c>
+      <c r="D39" s="16"/>
+      <c r="E39" s="17"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="18" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="53">
+  <mergeCells count="15">
+    <mergeCell ref="B34:B38"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B58:B62"/>
-    <mergeCell ref="B39:E39"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:B14"/>
@@ -2186,49 +1364,12 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:B50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B94:B98"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B100:B104"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="B106:B110"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B118:B122"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B124:B128"/>
-    <mergeCell ref="B142:B146"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:B152"/>
-    <mergeCell ref="B129:E129"/>
-    <mergeCell ref="B130:B134"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B136:B140"/>
-    <mergeCell ref="B141:E141"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C52:C56 C46:C50 C34:C38 C40:C44 C16:C20 B6 C22:C26 C28:C32 C58:C62 C148:C152 C6:C8 C76:C80 C82:C86 C70:C74 C64:C67 C88:C92 C94:C98 C100:C104 C106:C110 C112:C116 C118:C122 C124:C128 C130:C134 C136:C140 C142:C146 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C34:C38 C16:C20 B6 C22:C26 C28:C32 C6:C8 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B58:B62 B16:B20 B22:B26 B28:B32 B34:B38 B40:B44 B46:B50 B52:B56 B64:B68 B70:B74 B76:B80 B82:B86 B88:B92 B94:B98 B100:B104 B106:B110 B112:B116 B118:B122 B124:B128 B130:B134 B136:B140 B142:B146 B148:B152 B10:B14" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B16:B20 B22:B26 B28:B32 B34:B38 B10:B14" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2239,7 +1380,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="42" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2257,6 +1398,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -2438,15 +1588,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -2464,6 +1605,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2479,12 +1628,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : Mise a jour du jdt du 18.09.2026
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E26DA5E-83BC-4FF7-B824-BA89FFC5BE7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB8423F-9A52-43A5-BBB4-6B4866FD49F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="60">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -202,7 +202,34 @@
     <t>Début Projet</t>
   </si>
   <si>
-    <t>J'essaye de implémenter un joueur (classe, instanciation, image).</t>
+    <t>Erreur</t>
+  </si>
+  <si>
+    <t>J'ajoute la ressource du pirate (joueur) au projet et remplace fleet par joueur.</t>
+  </si>
+  <si>
+    <t>Je n'utilisais pas la bonne base, je recommence tout en ajoutant le joueur etc…</t>
+  </si>
+  <si>
+    <t>Mouvements</t>
+  </si>
+  <si>
+    <t>Je commence à ajouter un moyen de changer les mouvements avec le clavier.</t>
+  </si>
+  <si>
+    <t>Fonctionne mais le bas nombre de ups se fait ressentir.</t>
+  </si>
+  <si>
+    <t>Je change le mouvement pour que le joueur commence à bouger lentement puis accélère crescendo.</t>
+  </si>
+  <si>
+    <t>Tirs amis</t>
+  </si>
+  <si>
+    <t>Je plonge dans la création de classe gouvernail [WIP].</t>
+  </si>
+  <si>
+    <t>seulement ajouté classe et sprite.</t>
   </si>
 </sst>
 </file>
@@ -1187,7 +1214,7 @@
       </c>
       <c r="B21" s="36">
         <f>SUM(C22:C26)</f>
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="C21" s="37"/>
       <c r="D21" s="37"/>
@@ -1204,37 +1231,65 @@
         <v>60</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="27"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E22" s="27"/>
-    </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
       <c r="B23" s="34"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
+      <c r="C23" s="8">
+        <v>40</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
+      <c r="A24" s="7" t="s">
+        <v>53</v>
+      </c>
       <c r="B24" s="34"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="8"/>
+      <c r="C24" s="8">
+        <v>35</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
+      <c r="A25" s="7" t="s">
+        <v>53</v>
+      </c>
       <c r="B25" s="34"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
+      <c r="C25" s="8">
+        <v>30</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>56</v>
+      </c>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
+      <c r="A26" s="10" t="s">
+        <v>57</v>
+      </c>
       <c r="B26" s="35"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="10"/>
+      <c r="C26" s="10">
+        <v>15</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
@@ -1337,7 +1392,7 @@
       <c r="B39" s="26"/>
       <c r="C39" s="15">
         <f>MROUND(SUM(C6:C38) /60,0.2)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D39" s="16"/>
       <c r="E39" s="17"/>

</xml_diff>

<commit_message>
chore(jdt) : mise à jour du 25.09.2026
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB8423F-9A52-43A5-BBB4-6B4866FD49F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3FD8AC-7337-46DE-81F6-B3C4DF8788FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="67">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -230,6 +230,27 @@
   </si>
   <si>
     <t>seulement ajouté classe et sprite.</t>
+  </si>
+  <si>
+    <t>J'adapte le mouvement afin qu'il puisse toucher le bord et redevient lent en touchant le bord.</t>
+  </si>
+  <si>
+    <t>fond</t>
+  </si>
+  <si>
+    <t>J'ajoute une ressource qui servira de fond.</t>
+  </si>
+  <si>
+    <t>Gouvernail</t>
+  </si>
+  <si>
+    <t>J'essaye de créer une méthode mathhelpers pour la direction mais change d'avis, le gouvernail se fait simplement instancier et calcule lui-même la direction à partir de paramètres du constructeur.</t>
+  </si>
+  <si>
+    <t>Gouvernails</t>
+  </si>
+  <si>
+    <t>Je Continue l'implémentation, les projectiles sont instanciés justes et ont un cooldown.</t>
   </si>
 </sst>
 </file>
@@ -563,6 +584,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -574,18 +607,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -932,10 +953,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="29"/>
+      <c r="C1" s="32"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -947,10 +968,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="29"/>
+      <c r="C2" s="32"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -962,10 +983,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="29"/>
+      <c r="C3" s="32"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -977,12 +998,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="35"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1005,7 +1026,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="29">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1022,7 +1043,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="34"/>
+      <c r="B7" s="30"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1035,7 +1056,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="34"/>
+      <c r="B8" s="30"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1060,7 +1081,7 @@
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="33">
+      <c r="B10" s="29">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1075,7 +1096,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="34"/>
+      <c r="B11" s="30"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1088,7 +1109,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1101,7 +1122,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="34"/>
+      <c r="B13" s="30"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1114,7 +1135,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="35"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1141,7 +1162,7 @@
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="33">
+      <c r="B16" s="29">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1158,7 +1179,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="34"/>
+      <c r="B17" s="30"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1171,7 +1192,7 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="34"/>
+      <c r="B18" s="30"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
@@ -1186,7 +1207,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1199,7 +1220,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="35"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1224,7 +1245,7 @@
       <c r="A22" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="33">
+      <c r="B22" s="29">
         <v>46283</v>
       </c>
       <c r="C22" s="5">
@@ -1239,7 +1260,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="34"/>
+      <c r="B23" s="30"/>
       <c r="C23" s="8">
         <v>40</v>
       </c>
@@ -1252,7 +1273,7 @@
       <c r="A24" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="34"/>
+      <c r="B24" s="30"/>
       <c r="C24" s="8">
         <v>35</v>
       </c>
@@ -1267,7 +1288,7 @@
       <c r="A25" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="34"/>
+      <c r="B25" s="30"/>
       <c r="C25" s="8">
         <v>30</v>
       </c>
@@ -1280,7 +1301,7 @@
       <c r="A26" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B26" s="35"/>
+      <c r="B26" s="31"/>
       <c r="C26" s="10">
         <v>15</v>
       </c>
@@ -1297,43 +1318,69 @@
       </c>
       <c r="B27" s="36">
         <f>SUM(C28:C32)</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="C27" s="37"/>
       <c r="D27" s="37"/>
       <c r="E27" s="38"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="14"/>
+      <c r="A28" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="29">
+        <v>46290</v>
+      </c>
+      <c r="C28" s="13">
+        <v>30</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>60</v>
+      </c>
       <c r="E28" s="27"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
+      <c r="A29" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="30"/>
+      <c r="C29" s="8">
+        <v>10</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="E29" s="27"/>
     </row>
-    <row r="30" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="8"/>
-      <c r="B30" s="34"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
+    <row r="30" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="30"/>
+      <c r="C30" s="8">
+        <v>80</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>64</v>
+      </c>
       <c r="E30" s="27"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="8"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="9"/>
+      <c r="A31" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="30"/>
+      <c r="C31" s="8">
+        <v>60</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="35"/>
+      <c r="B32" s="31"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1352,35 +1399,35 @@
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="33"/>
+      <c r="B34" s="29"/>
       <c r="C34" s="5"/>
       <c r="D34" s="6"/>
       <c r="E34" s="27"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="34"/>
+      <c r="B35" s="30"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="27"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="34"/>
+      <c r="B36" s="30"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="27"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="34"/>
+      <c r="B37" s="30"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="35"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
@@ -1392,7 +1439,7 @@
       <c r="B39" s="26"/>
       <c r="C39" s="15">
         <f>MROUND(SUM(C6:C38) /60,0.2)</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D39" s="16"/>
       <c r="E39" s="17"/>
@@ -1453,15 +1500,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -1643,6 +1681,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1660,14 +1707,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1683,4 +1722,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : maj du 28.09.26
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -5,18 +5,18 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3FD8AC-7337-46DE-81F6-B3C4DF8788FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1930302E-5151-4451-A845-7E0330425BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$51</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="73">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -251,6 +251,24 @@
   </si>
   <si>
     <t>Je Continue l'implémentation, les projectiles sont instanciés justes et ont un cooldown.</t>
+  </si>
+  <si>
+    <t>Position juste</t>
+  </si>
+  <si>
+    <t>J'essaye d'adapter la position x et y au centre du joueur mais laisse tomber car le besoin n'est pas vraiment là.</t>
+  </si>
+  <si>
+    <t>Je lis le code qui sert à render le GameSpace afin de comprendre comment changer de fond.</t>
+  </si>
+  <si>
+    <t>Analyse</t>
+  </si>
+  <si>
+    <t>Obstacles</t>
+  </si>
+  <si>
+    <t>Début de la création de la classe Obstacle.</t>
   </si>
 </sst>
 </file>
@@ -936,17 +954,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E53"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="107" style="1" customWidth="1"/>
-    <col min="5" max="5" width="71.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="71.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="1"/>
+    <col min="8" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1022,7 +1040,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
@@ -1039,7 +1057,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
@@ -1131,7 +1149,7 @@
       </c>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
@@ -1391,31 +1409,51 @@
       </c>
       <c r="B33" s="36">
         <f>SUM(C34:C38)</f>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C33" s="37"/>
       <c r="D33" s="37"/>
       <c r="E33" s="38"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6"/>
+      <c r="A34" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" s="29">
+        <v>46293</v>
+      </c>
+      <c r="C34" s="5">
+        <v>15</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="E34" s="27"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
+      <c r="A35" s="7" t="s">
+        <v>70</v>
+      </c>
       <c r="B35" s="30"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
+      <c r="C35" s="8">
+        <v>10</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>69</v>
+      </c>
       <c r="E35" s="27"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
+      <c r="A36" s="7" t="s">
+        <v>71</v>
+      </c>
       <c r="B36" s="30"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
+      <c r="C36" s="8">
+        <v>10</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="E36" s="27"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1432,25 +1470,123 @@
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
     </row>
-    <row r="39" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="25" t="s">
+    <row r="39" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B39" s="36">
+        <f>SUM(C40:C44)</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="38"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="4"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="27"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="7"/>
+      <c r="B41" s="30"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="27"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="7"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="27"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="7"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="8"/>
+    </row>
+    <row r="44" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="10"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="10"/>
+    </row>
+    <row r="45" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="36">
+        <f>SUM(C46:C50)</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="4"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="27"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="7"/>
+      <c r="B47" s="30"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="27"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="7"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="27"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="7"/>
+      <c r="B49" s="30"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="10"/>
+      <c r="B50" s="31"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="10"/>
+    </row>
+    <row r="51" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B39" s="26"/>
-      <c r="C39" s="15">
+      <c r="B51" s="26"/>
+      <c r="C51" s="15">
         <f>MROUND(SUM(C6:C38) /60,0.2)</f>
-        <v>15</v>
-      </c>
-      <c r="D39" s="16"/>
-      <c r="E39" s="17"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="18" t="s">
+        <v>15.600000000000001</v>
+      </c>
+      <c r="D51" s="16"/>
+      <c r="E51" s="17"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="18" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="19">
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:B50"/>
     <mergeCell ref="B34:B38"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1468,10 +1604,10 @@
     <mergeCell ref="B33:E33"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C34:C38 C16:C20 B6 C22:C26 C28:C32 C6:C8 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C34:C38 C16:C20 B6 C22:C26 C28:C32 C6:C8 C10:C14 C40:C44 C46:C50" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B16:B20 B22:B26 B28:B32 B34:B38 B10:B14" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B16:B20 B22:B26 B28:B32 B46:B50 B10:B14 B40:B44 B34:B38" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1482,7 +1618,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="42" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="40" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1500,6 +1636,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -1681,15 +1826,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -1707,6 +1843,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1722,12 +1866,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : Maj du jdt pour le 04.10.2026
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1930302E-5151-4451-A845-7E0330425BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97A3A30D-B526-40CE-88AD-AA9B5F9FEE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$153</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="59">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -199,83 +199,41 @@
     <t>Le Cdp commente ma release v1 et me dis ce qui est à revoir.</t>
   </si>
   <si>
-    <t>Début Projet</t>
-  </si>
-  <si>
-    <t>Erreur</t>
-  </si>
-  <si>
-    <t>J'ajoute la ressource du pirate (joueur) au projet et remplace fleet par joueur.</t>
-  </si>
-  <si>
-    <t>Je n'utilisais pas la bonne base, je recommence tout en ajoutant le joueur etc…</t>
-  </si>
-  <si>
-    <t>Mouvements</t>
-  </si>
-  <si>
-    <t>Je commence à ajouter un moyen de changer les mouvements avec le clavier.</t>
-  </si>
-  <si>
-    <t>Fonctionne mais le bas nombre de ups se fait ressentir.</t>
-  </si>
-  <si>
-    <t>Je change le mouvement pour que le joueur commence à bouger lentement puis accélère crescendo.</t>
-  </si>
-  <si>
-    <t>Tirs amis</t>
-  </si>
-  <si>
-    <t>Je plonge dans la création de classe gouvernail [WIP].</t>
-  </si>
-  <si>
-    <t>seulement ajouté classe et sprite.</t>
-  </si>
-  <si>
-    <t>J'adapte le mouvement afin qu'il puisse toucher le bord et redevient lent en touchant le bord.</t>
-  </si>
-  <si>
-    <t>fond</t>
-  </si>
-  <si>
-    <t>J'ajoute une ressource qui servira de fond.</t>
-  </si>
-  <si>
-    <t>Gouvernail</t>
-  </si>
-  <si>
-    <t>J'essaye de créer une méthode mathhelpers pour la direction mais change d'avis, le gouvernail se fait simplement instancier et calcule lui-même la direction à partir de paramètres du constructeur.</t>
-  </si>
-  <si>
-    <t>Gouvernails</t>
-  </si>
-  <si>
-    <t>Je Continue l'implémentation, les projectiles sont instanciés justes et ont un cooldown.</t>
-  </si>
-  <si>
-    <t>Position juste</t>
-  </si>
-  <si>
-    <t>J'essaye d'adapter la position x et y au centre du joueur mais laisse tomber car le besoin n'est pas vraiment là.</t>
-  </si>
-  <si>
-    <t>Je lis le code qui sert à render le GameSpace afin de comprendre comment changer de fond.</t>
-  </si>
-  <si>
-    <t>Analyse</t>
-  </si>
-  <si>
-    <t>Obstacles</t>
-  </si>
-  <si>
-    <t>Début de la création de la classe Obstacle.</t>
+    <t>Je finis rapidement un point du module.</t>
+  </si>
+  <si>
+    <t>Sprite</t>
+  </si>
+  <si>
+    <t>Je fais un dessin vite fais pour les 4 états de obstacle.</t>
+  </si>
+  <si>
+    <t>Obstacle</t>
+  </si>
+  <si>
+    <t>J'avance sur obstacles, j'essaye de leur donner 4 états avec une image différente, je refais les images 2 fois.</t>
+  </si>
+  <si>
+    <t>Je crée une méthode dans MathHelpers pour détecter les collisions (IsTouching) et détecte les collisions entre gouvernails et obstacles avec.</t>
+  </si>
+  <si>
+    <t>Collisions</t>
+  </si>
+  <si>
+    <t>Je finis les obstacles</t>
+  </si>
+  <si>
+    <t>Ennemi</t>
+  </si>
+  <si>
+    <t>Je commence les ennemis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Century Gothic"/>
@@ -325,6 +283,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Century Gothic"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -508,7 +472,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -591,6 +555,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -598,10 +563,26 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -614,28 +595,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -954,7 +931,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6640625" style="1" customWidth="1"/>
@@ -971,10 +948,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32"/>
+      <c r="C1" s="31"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -986,10 +963,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="32"/>
+      <c r="C2" s="31"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1001,10 +978,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="32"/>
+      <c r="C3" s="31"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1016,12 +993,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="35"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1044,7 +1021,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="35">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1061,7 +1038,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="30"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1074,7 +1051,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="30"/>
+      <c r="B8" s="36"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1087,19 +1064,16 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="36">
-        <f>SUM(C10:C14)</f>
-        <v>180</v>
-      </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="38"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="40"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="29">
+      <c r="B10" s="35">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1108,13 +1082,13 @@
       <c r="D10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="27"/>
+      <c r="E10" s="28"/>
     </row>
     <row r="11" spans="1:5" s="23" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="30"/>
+      <c r="B11" s="36"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1127,7 +1101,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="30"/>
+      <c r="B12" s="36"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1140,7 +1114,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="30"/>
+      <c r="B13" s="36"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1153,7 +1127,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="31"/>
+      <c r="B14" s="37"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1168,19 +1142,16 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="36">
-        <f>SUM(C16:C20)</f>
-        <v>180</v>
-      </c>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="38"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="40"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="29">
+      <c r="B16" s="35">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1189,7 +1160,7 @@
       <c r="D16" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="28" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1197,7 +1168,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="30"/>
+      <c r="B17" s="36"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1210,14 +1181,14 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="30"/>
+      <c r="B18" s="36"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="30" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1225,7 +1196,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="30"/>
+      <c r="B19" s="36"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1238,7 +1209,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="31"/>
+      <c r="B20" s="37"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1251,154 +1222,126 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="36">
-        <f>SUM(C22:C26)</f>
-        <v>180</v>
-      </c>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="40"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="4">
+        <v>320</v>
+      </c>
+      <c r="B22" s="35">
+        <v>46297</v>
+      </c>
+      <c r="C22" s="5">
+        <v>5</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="29">
-        <v>46283</v>
-      </c>
-      <c r="C22" s="5">
-        <v>60</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="28"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="30"/>
+      <c r="B23" s="36"/>
       <c r="C23" s="8">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="36"/>
+      <c r="C24" s="8">
+        <v>160</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="8">
-        <v>35</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>55</v>
-      </c>
+      <c r="E24" s="8"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="30"/>
-      <c r="C25" s="8">
-        <v>30</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>56</v>
-      </c>
+      <c r="A25" s="7"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="10">
-        <v>15</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>59</v>
-      </c>
+      <c r="A26" s="10"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="10"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="36">
-        <f>SUM(C28:C32)</f>
-        <v>180</v>
-      </c>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38"/>
-    </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="38"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="40"/>
+    </row>
+    <row r="28" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="29">
-        <v>46290</v>
+        <v>52</v>
+      </c>
+      <c r="B28" s="35">
+        <v>46299</v>
       </c>
       <c r="C28" s="13">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" s="27"/>
-    </row>
-    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="E28" s="28"/>
+    </row>
+    <row r="29" spans="1:5" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B29" s="30"/>
+        <v>55</v>
+      </c>
+      <c r="B29" s="36"/>
       <c r="C29" s="8">
+        <v>70</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E29" s="28"/>
+    </row>
+    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="36"/>
+      <c r="C30" s="8">
         <v>10</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="E29" s="27"/>
-    </row>
-    <row r="30" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="8">
-        <v>80</v>
-      </c>
       <c r="D30" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E30" s="27"/>
+        <v>58</v>
+      </c>
+      <c r="E30" s="28"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B31" s="30"/>
-      <c r="C31" s="8">
-        <v>60</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>66</v>
-      </c>
+      <c r="A31" s="8"/>
+      <c r="B31" s="36"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="31"/>
+      <c r="B32" s="37"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1407,191 +1350,939 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="36">
-        <f>SUM(C34:C38)</f>
-        <v>35</v>
-      </c>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="38"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="40"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" s="29">
-        <v>46293</v>
-      </c>
-      <c r="C34" s="5">
-        <v>15</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E34" s="27"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="35"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="28"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B35" s="30"/>
-      <c r="C35" s="8">
-        <v>10</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E35" s="27"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="28"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="8">
-        <v>10</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E36" s="27"/>
+      <c r="A36" s="7"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="28"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="30"/>
+      <c r="B37" s="36"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
-      <c r="B38" s="31"/>
+      <c r="B38" s="37"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
     </row>
-    <row r="39" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="36">
-        <f>SUM(C40:C44)</f>
-        <v>0</v>
-      </c>
-      <c r="C39" s="37"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="38"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B39" s="38"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="40"/>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
-      <c r="B40" s="29"/>
+      <c r="B40" s="35"/>
       <c r="C40" s="5"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="27"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D40" s="25"/>
+      <c r="E40" s="5"/>
+    </row>
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7"/>
-      <c r="B41" s="30"/>
+      <c r="B41" s="36"/>
       <c r="C41" s="8"/>
       <c r="D41" s="9"/>
-      <c r="E41" s="27"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="28"/>
+    </row>
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
-      <c r="B42" s="30"/>
+      <c r="B42" s="36"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
-      <c r="E42" s="27"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="28"/>
+    </row>
+    <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="30"/>
+      <c r="B43" s="36"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
-    <row r="44" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="31"/>
+      <c r="B44" s="37"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
     </row>
-    <row r="45" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B45" s="36">
-        <f>SUM(C46:C50)</f>
-        <v>0</v>
-      </c>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="12"/>
+      <c r="B45" s="38"/>
+      <c r="C45" s="39"/>
+      <c r="D45" s="39"/>
+      <c r="E45" s="40"/>
+    </row>
+    <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
-      <c r="B46" s="29"/>
+      <c r="B46" s="35"/>
       <c r="C46" s="5"/>
       <c r="D46" s="6"/>
-      <c r="E46" s="27"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="28"/>
+    </row>
+    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
-      <c r="B47" s="30"/>
+      <c r="B47" s="36"/>
       <c r="C47" s="8"/>
       <c r="D47" s="9"/>
-      <c r="E47" s="27"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="28"/>
+    </row>
+    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="30"/>
+      <c r="B48" s="36"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
-      <c r="E48" s="27"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="30"/>
+      <c r="B49" s="36"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
-    <row r="50" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="10"/>
-      <c r="B50" s="31"/>
+      <c r="B50" s="37"/>
       <c r="C50" s="10"/>
       <c r="D50" s="11"/>
       <c r="E50" s="10"/>
     </row>
-    <row r="51" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="25" t="s">
+    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="38"/>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="40"/>
+    </row>
+    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="4"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="28"/>
+    </row>
+    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="36"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="28"/>
+    </row>
+    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="36"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="8"/>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="7"/>
+      <c r="B55" s="36"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="8"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="10"/>
+      <c r="B56" s="37"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="10"/>
+    </row>
+    <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B57" s="38"/>
+      <c r="C57" s="39"/>
+      <c r="D57" s="39"/>
+      <c r="E57" s="40"/>
+    </row>
+    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="13"/>
+      <c r="B58" s="35"/>
+      <c r="C58" s="13"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="28"/>
+    </row>
+    <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="8"/>
+      <c r="B59" s="36"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="28"/>
+    </row>
+    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="8"/>
+      <c r="B60" s="36"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="8"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="8"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="8"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="8"/>
+      <c r="B62" s="37"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="8"/>
+    </row>
+    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B63" s="38"/>
+      <c r="C63" s="39"/>
+      <c r="D63" s="39"/>
+      <c r="E63" s="40"/>
+    </row>
+    <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="8"/>
+      <c r="B64" s="35"/>
+      <c r="C64" s="13"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="28"/>
+    </row>
+    <row r="65" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="36"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="8"/>
+    </row>
+    <row r="66" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="8"/>
+      <c r="B66" s="36"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="8"/>
+    </row>
+    <row r="67" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="8"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="8"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="8"/>
+      <c r="B68" s="37"/>
+      <c r="E68" s="8"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B69" s="38"/>
+      <c r="C69" s="39"/>
+      <c r="D69" s="39"/>
+      <c r="E69" s="40"/>
+    </row>
+    <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="8"/>
+      <c r="B70" s="35"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="28"/>
+    </row>
+    <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="8"/>
+      <c r="B71" s="36"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="8"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="8"/>
+      <c r="B72" s="36"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="8"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="8"/>
+      <c r="B73" s="36"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="8"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="8"/>
+      <c r="B74" s="37"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="8"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B75" s="38"/>
+      <c r="C75" s="39"/>
+      <c r="D75" s="39"/>
+      <c r="E75" s="40"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="13"/>
+      <c r="B76" s="35"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="14"/>
+      <c r="E76" s="28"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="8"/>
+      <c r="B77" s="36"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="8"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="8"/>
+      <c r="B78" s="36"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="29"/>
+      <c r="E78" s="8"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="8"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="9"/>
+      <c r="E79" s="8"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="8"/>
+      <c r="B80" s="37"/>
+      <c r="C80" s="8"/>
+      <c r="D80" s="9"/>
+      <c r="E80" s="8"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B81" s="38"/>
+      <c r="C81" s="39"/>
+      <c r="D81" s="39"/>
+      <c r="E81" s="40"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="13"/>
+      <c r="B82" s="35"/>
+      <c r="C82" s="13"/>
+      <c r="D82" s="14"/>
+      <c r="E82" s="28"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="13"/>
+      <c r="B83" s="41"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="14"/>
+      <c r="E83" s="28"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="8"/>
+      <c r="B84" s="41"/>
+      <c r="C84" s="8"/>
+      <c r="D84" s="9"/>
+      <c r="E84" s="8"/>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="8"/>
+      <c r="B85" s="41"/>
+      <c r="C85" s="8"/>
+      <c r="D85" s="9"/>
+      <c r="E85" s="8"/>
+    </row>
+    <row r="86" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="8"/>
+      <c r="B86" s="42"/>
+      <c r="C86" s="8"/>
+      <c r="D86" s="9"/>
+      <c r="E86" s="8"/>
+    </row>
+    <row r="87" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B87" s="38"/>
+      <c r="C87" s="39"/>
+      <c r="D87" s="39"/>
+      <c r="E87" s="40"/>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="13"/>
+      <c r="B88" s="35"/>
+      <c r="C88" s="13"/>
+      <c r="D88" s="14"/>
+      <c r="E88" s="28"/>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="13"/>
+      <c r="B89" s="41"/>
+      <c r="C89" s="8"/>
+      <c r="D89" s="14"/>
+      <c r="E89" s="28"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="8"/>
+      <c r="B90" s="41"/>
+      <c r="C90" s="8"/>
+      <c r="D90" s="9"/>
+      <c r="E90" s="8"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="8"/>
+      <c r="B91" s="41"/>
+      <c r="C91" s="8"/>
+      <c r="D91" s="9"/>
+      <c r="E91" s="8"/>
+    </row>
+    <row r="92" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="8"/>
+      <c r="B92" s="42"/>
+      <c r="C92" s="8"/>
+      <c r="D92" s="9"/>
+      <c r="E92" s="8"/>
+    </row>
+    <row r="93" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B93" s="38"/>
+      <c r="C93" s="39"/>
+      <c r="D93" s="39"/>
+      <c r="E93" s="40"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="13"/>
+      <c r="B94" s="35"/>
+      <c r="C94" s="13"/>
+      <c r="D94" s="14"/>
+      <c r="E94" s="28"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="13"/>
+      <c r="B95" s="41"/>
+      <c r="C95" s="8"/>
+      <c r="D95" s="14"/>
+      <c r="E95" s="28"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="8"/>
+      <c r="B96" s="41"/>
+      <c r="C96" s="8"/>
+      <c r="D96" s="9"/>
+      <c r="E96" s="8"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="8"/>
+      <c r="B97" s="41"/>
+      <c r="C97" s="8"/>
+      <c r="D97" s="9"/>
+      <c r="E97" s="8"/>
+    </row>
+    <row r="98" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="8"/>
+      <c r="B98" s="42"/>
+      <c r="C98" s="8"/>
+      <c r="D98" s="9"/>
+      <c r="E98" s="8"/>
+    </row>
+    <row r="99" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B99" s="38"/>
+      <c r="C99" s="39"/>
+      <c r="D99" s="39"/>
+      <c r="E99" s="40"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="13"/>
+      <c r="B100" s="35"/>
+      <c r="C100" s="13"/>
+      <c r="D100" s="14"/>
+      <c r="E100" s="28"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="13"/>
+      <c r="B101" s="41"/>
+      <c r="C101" s="8"/>
+      <c r="D101" s="14"/>
+      <c r="E101" s="28"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="8"/>
+      <c r="B102" s="41"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="9"/>
+      <c r="E102" s="8"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="8"/>
+      <c r="B103" s="41"/>
+      <c r="C103" s="8"/>
+      <c r="D103" s="9"/>
+      <c r="E103" s="8"/>
+    </row>
+    <row r="104" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="8"/>
+      <c r="B104" s="42"/>
+      <c r="C104" s="8"/>
+      <c r="D104" s="9"/>
+      <c r="E104" s="8"/>
+    </row>
+    <row r="105" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B105" s="38"/>
+      <c r="C105" s="39"/>
+      <c r="D105" s="39"/>
+      <c r="E105" s="40"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="13"/>
+      <c r="B106" s="35"/>
+      <c r="C106" s="13"/>
+      <c r="D106" s="14"/>
+      <c r="E106" s="28"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="13"/>
+      <c r="B107" s="41"/>
+      <c r="C107" s="8"/>
+      <c r="D107" s="14"/>
+      <c r="E107" s="28"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="8"/>
+      <c r="B108" s="41"/>
+      <c r="C108" s="8"/>
+      <c r="D108" s="9"/>
+      <c r="E108" s="8"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="8"/>
+      <c r="B109" s="41"/>
+      <c r="C109" s="8"/>
+      <c r="D109" s="9"/>
+      <c r="E109" s="8"/>
+    </row>
+    <row r="110" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="8"/>
+      <c r="B110" s="42"/>
+      <c r="C110" s="8"/>
+      <c r="D110" s="9"/>
+      <c r="E110" s="8"/>
+    </row>
+    <row r="111" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B111" s="38"/>
+      <c r="C111" s="39"/>
+      <c r="D111" s="39"/>
+      <c r="E111" s="40"/>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="13"/>
+      <c r="B112" s="35"/>
+      <c r="C112" s="13"/>
+      <c r="D112" s="14"/>
+      <c r="E112" s="28"/>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="13"/>
+      <c r="B113" s="41"/>
+      <c r="C113" s="8"/>
+      <c r="D113" s="14"/>
+      <c r="E113" s="28"/>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="8"/>
+      <c r="B114" s="41"/>
+      <c r="C114" s="8"/>
+      <c r="D114" s="9"/>
+      <c r="E114" s="8"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="8"/>
+      <c r="B115" s="41"/>
+      <c r="C115" s="8"/>
+      <c r="D115" s="9"/>
+      <c r="E115" s="8"/>
+    </row>
+    <row r="116" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="8"/>
+      <c r="B116" s="42"/>
+      <c r="C116" s="8"/>
+      <c r="D116" s="9"/>
+      <c r="E116" s="8"/>
+    </row>
+    <row r="117" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B117" s="38"/>
+      <c r="C117" s="39"/>
+      <c r="D117" s="39"/>
+      <c r="E117" s="40"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="13"/>
+      <c r="B118" s="35"/>
+      <c r="C118" s="13"/>
+      <c r="D118" s="14"/>
+      <c r="E118" s="28"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" s="13"/>
+      <c r="B119" s="41"/>
+      <c r="C119" s="8"/>
+      <c r="D119" s="14"/>
+      <c r="E119" s="28"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" s="8"/>
+      <c r="B120" s="41"/>
+      <c r="C120" s="8"/>
+      <c r="D120" s="9"/>
+      <c r="E120" s="8"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" s="8"/>
+      <c r="B121" s="41"/>
+      <c r="C121" s="8"/>
+      <c r="D121" s="9"/>
+      <c r="E121" s="8"/>
+    </row>
+    <row r="122" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="8"/>
+      <c r="B122" s="42"/>
+      <c r="C122" s="8"/>
+      <c r="D122" s="9"/>
+      <c r="E122" s="8"/>
+    </row>
+    <row r="123" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B123" s="38"/>
+      <c r="C123" s="39"/>
+      <c r="D123" s="39"/>
+      <c r="E123" s="40"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" s="13"/>
+      <c r="B124" s="35"/>
+      <c r="C124" s="13"/>
+      <c r="D124" s="14"/>
+      <c r="E124" s="28"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" s="13"/>
+      <c r="B125" s="41"/>
+      <c r="C125" s="8"/>
+      <c r="D125" s="14"/>
+      <c r="E125" s="28"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" s="8"/>
+      <c r="B126" s="41"/>
+      <c r="C126" s="8"/>
+      <c r="D126" s="9"/>
+      <c r="E126" s="8"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" s="8"/>
+      <c r="B127" s="41"/>
+      <c r="C127" s="8"/>
+      <c r="D127" s="9"/>
+      <c r="E127" s="8"/>
+    </row>
+    <row r="128" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="8"/>
+      <c r="B128" s="42"/>
+      <c r="C128" s="8"/>
+      <c r="D128" s="9"/>
+      <c r="E128" s="8"/>
+    </row>
+    <row r="129" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B129" s="38"/>
+      <c r="C129" s="39"/>
+      <c r="D129" s="39"/>
+      <c r="E129" s="40"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" s="13"/>
+      <c r="B130" s="35"/>
+      <c r="C130" s="13"/>
+      <c r="D130" s="14"/>
+      <c r="E130" s="28"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" s="13"/>
+      <c r="B131" s="41"/>
+      <c r="C131" s="8"/>
+      <c r="D131" s="14"/>
+      <c r="E131" s="28"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" s="8"/>
+      <c r="B132" s="41"/>
+      <c r="C132" s="8"/>
+      <c r="D132" s="9"/>
+      <c r="E132" s="8"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" s="8"/>
+      <c r="B133" s="41"/>
+      <c r="C133" s="8"/>
+      <c r="D133" s="9"/>
+      <c r="E133" s="8"/>
+    </row>
+    <row r="134" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="8"/>
+      <c r="B134" s="42"/>
+      <c r="C134" s="8"/>
+      <c r="D134" s="9"/>
+      <c r="E134" s="8"/>
+    </row>
+    <row r="135" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B135" s="38"/>
+      <c r="C135" s="39"/>
+      <c r="D135" s="39"/>
+      <c r="E135" s="40"/>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" s="13"/>
+      <c r="B136" s="35"/>
+      <c r="C136" s="13"/>
+      <c r="D136" s="14"/>
+      <c r="E136" s="28"/>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" s="13"/>
+      <c r="B137" s="41"/>
+      <c r="C137" s="8"/>
+      <c r="D137" s="14"/>
+      <c r="E137" s="28"/>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" s="8"/>
+      <c r="B138" s="41"/>
+      <c r="C138" s="8"/>
+      <c r="D138" s="9"/>
+      <c r="E138" s="8"/>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" s="8"/>
+      <c r="B139" s="41"/>
+      <c r="C139" s="8"/>
+      <c r="D139" s="9"/>
+      <c r="E139" s="8"/>
+    </row>
+    <row r="140" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="8"/>
+      <c r="B140" s="42"/>
+      <c r="C140" s="8"/>
+      <c r="D140" s="9"/>
+      <c r="E140" s="8"/>
+    </row>
+    <row r="141" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B141" s="38"/>
+      <c r="C141" s="39"/>
+      <c r="D141" s="39"/>
+      <c r="E141" s="40"/>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" s="13"/>
+      <c r="B142" s="35"/>
+      <c r="C142" s="13"/>
+      <c r="D142" s="14"/>
+      <c r="E142" s="28"/>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" s="13"/>
+      <c r="B143" s="41"/>
+      <c r="C143" s="8"/>
+      <c r="D143" s="14"/>
+      <c r="E143" s="28"/>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" s="8"/>
+      <c r="B144" s="41"/>
+      <c r="C144" s="8"/>
+      <c r="D144" s="9"/>
+      <c r="E144" s="8"/>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" s="8"/>
+      <c r="B145" s="41"/>
+      <c r="C145" s="8"/>
+      <c r="D145" s="9"/>
+      <c r="E145" s="8"/>
+    </row>
+    <row r="146" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="8"/>
+      <c r="B146" s="42"/>
+      <c r="C146" s="8"/>
+      <c r="D146" s="9"/>
+      <c r="E146" s="8"/>
+    </row>
+    <row r="147" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B147" s="38"/>
+      <c r="C147" s="39"/>
+      <c r="D147" s="39"/>
+      <c r="E147" s="40"/>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" s="13"/>
+      <c r="B148" s="35"/>
+      <c r="C148" s="13"/>
+      <c r="D148" s="14"/>
+      <c r="E148" s="28"/>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" s="13"/>
+      <c r="B149" s="41"/>
+      <c r="C149" s="8"/>
+      <c r="D149" s="14"/>
+      <c r="E149" s="28"/>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" s="8"/>
+      <c r="B150" s="41"/>
+      <c r="C150" s="8"/>
+      <c r="D150" s="9"/>
+      <c r="E150" s="8"/>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="8"/>
+      <c r="B151" s="41"/>
+      <c r="C151" s="8"/>
+      <c r="D151" s="9"/>
+      <c r="E151" s="8"/>
+    </row>
+    <row r="152" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="8"/>
+      <c r="B152" s="42"/>
+      <c r="C152" s="8"/>
+      <c r="D152" s="9"/>
+      <c r="E152" s="8"/>
+    </row>
+    <row r="153" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="26"/>
-      <c r="C51" s="15">
-        <f>MROUND(SUM(C6:C38) /60,0.2)</f>
-        <v>15.600000000000001</v>
-      </c>
-      <c r="D51" s="16"/>
-      <c r="E51" s="17"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="18" t="s">
+      <c r="B153" s="27"/>
+      <c r="C153" s="15">
+        <f>MROUND(SUM(C6:C152) /60,0.2)</f>
+        <v>13.600000000000001</v>
+      </c>
+      <c r="D153" s="16"/>
+      <c r="E153" s="17"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" s="18" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B39:E39"/>
+  <mergeCells count="53">
+    <mergeCell ref="B142:B146"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:B152"/>
+    <mergeCell ref="B129:E129"/>
+    <mergeCell ref="B130:B134"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B136:B140"/>
+    <mergeCell ref="B141:E141"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B118:B122"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B124:B128"/>
+    <mergeCell ref="B100:B104"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="B106:B110"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B88:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B94:B98"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B34:B38"/>
     <mergeCell ref="B40:B44"/>
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B46:B50"/>
-    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="B76:B80"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B58:B62"/>
+    <mergeCell ref="B39:E39"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:B14"/>
@@ -1604,10 +2295,10 @@
     <mergeCell ref="B33:E33"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C34:C38 C16:C20 B6 C22:C26 C28:C32 C6:C8 C10:C14 C40:C44 C46:C50" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C52:C56 C46:C50 C34:C38 C40:C44 C16:C20 B6 C22:C26 C28:C32 C58:C62 C148:C152 C6:C8 C76:C80 C82:C86 C70:C74 C64:C67 C88:C92 C94:C98 C100:C104 C106:C110 C112:C116 C118:C122 C124:C128 C130:C134 C136:C140 C142:C146 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B16:B20 B22:B26 B28:B32 B46:B50 B10:B14 B40:B44 B34:B38" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B58:B62 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B46:B50 B52:B56 B64:B68 B70:B74 B76:B80 B82:B86 B88:B92 B94:B98 B100:B104 B106:B110 B112:B116 B118:B122 B124:B128 B130:B134 B136:B140 B142:B146 B148:B152 B28:B32" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1618,7 +2309,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="40" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="30" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1829,15 +2520,15 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
chore(jdt) : maj du 09.10.26
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97A3A30D-B526-40CE-88AD-AA9B5F9FEE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD8CC72-867B-4EAE-9A54-2BABF2ADE9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="68">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -227,6 +227,33 @@
   </si>
   <si>
     <t>Je commence les ennemis</t>
+  </si>
+  <si>
+    <t>Je travaille sur la classe ennemi</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>Je crée une classe location pour simplifier la lecture (j'avais des tableaux 2d avant)</t>
+  </si>
+  <si>
+    <t>sprites</t>
+  </si>
+  <si>
+    <t>je travaille sur des sprites pour les ennemis et améliore legèrement le pirate.</t>
+  </si>
+  <si>
+    <t>renommage solution</t>
+  </si>
+  <si>
+    <t>J'essaye de renommer la solution et le projet mais J'ai trop de problême, j'opte pour avancer le 80% plutôt.</t>
+  </si>
+  <si>
+    <t>Autres</t>
+  </si>
+  <si>
+    <t>Je fais des commentaires dans presque tout les fichiers, ajoute des rndHelpers et commente.</t>
   </si>
 </sst>
 </file>
@@ -932,16 +959,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E155"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="107" style="1" customWidth="1"/>
-    <col min="5" max="5" width="71.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="71.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.44140625" style="1"/>
+    <col min="8" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1017,7 +1044,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
@@ -1034,7 +1061,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
@@ -1123,7 +1150,7 @@
       </c>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
@@ -1291,7 +1318,7 @@
       <c r="D27" s="39"/>
       <c r="E27" s="40"/>
     </row>
-    <row r="28" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
@@ -1355,39 +1382,71 @@
       <c r="D33" s="39"/>
       <c r="E33" s="40"/>
     </row>
-    <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6"/>
+    <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="35">
+        <v>46304</v>
+      </c>
+      <c r="C34" s="5">
+        <v>20</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>63</v>
+      </c>
       <c r="E34" s="28"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
+      <c r="A35" s="4" t="s">
+        <v>57</v>
+      </c>
       <c r="B35" s="36"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
+      <c r="C35" s="5">
+        <v>160</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="E35" s="28"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
+      <c r="A36" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="B36" s="36"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
+      <c r="C36" s="8">
+        <v>5</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>61</v>
+      </c>
       <c r="E36" s="28"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
+      <c r="A37" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="B37" s="36"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
+      <c r="C37" s="8">
+        <v>15</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>65</v>
+      </c>
       <c r="E37" s="8"/>
     </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10"/>
+    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="10" t="s">
+        <v>66</v>
+      </c>
       <c r="B38" s="37"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="11"/>
+      <c r="C38" s="10">
+        <v>20</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>67</v>
+      </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1434,8 +1493,10 @@
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
     </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="12"/>
+    <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="B45" s="38"/>
       <c r="C45" s="39"/>
       <c r="D45" s="39"/>
@@ -1476,7 +1537,7 @@
       <c r="D50" s="11"/>
       <c r="E50" s="10"/>
     </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
         <v>15</v>
       </c>
@@ -1557,14 +1618,14 @@
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="8"/>
       <c r="B62" s="37"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="12" t="s">
         <v>15</v>
       </c>
@@ -1606,9 +1667,7 @@
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="A69" s="12"/>
       <c r="B69" s="38"/>
       <c r="C69" s="39"/>
       <c r="D69" s="39"/>
@@ -1650,9 +1709,7 @@
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="A75" s="12"/>
       <c r="B75" s="38"/>
       <c r="C75" s="39"/>
       <c r="D75" s="39"/>
@@ -1694,9 +1751,7 @@
       <c r="E80" s="8"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="A81" s="12"/>
       <c r="B81" s="38"/>
       <c r="C81" s="39"/>
       <c r="D81" s="39"/>
@@ -1730,17 +1785,15 @@
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
-    <row r="86" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="8"/>
       <c r="B86" s="42"/>
       <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
-    <row r="87" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="12"/>
       <c r="B87" s="38"/>
       <c r="C87" s="39"/>
       <c r="D87" s="39"/>
@@ -1774,17 +1827,15 @@
       <c r="D91" s="9"/>
       <c r="E91" s="8"/>
     </row>
-    <row r="92" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="8"/>
       <c r="B92" s="42"/>
       <c r="C92" s="8"/>
       <c r="D92" s="9"/>
       <c r="E92" s="8"/>
     </row>
-    <row r="93" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="93" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="12"/>
       <c r="B93" s="38"/>
       <c r="C93" s="39"/>
       <c r="D93" s="39"/>
@@ -1818,17 +1869,15 @@
       <c r="D97" s="9"/>
       <c r="E97" s="8"/>
     </row>
-    <row r="98" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="8"/>
       <c r="B98" s="42"/>
       <c r="C98" s="8"/>
       <c r="D98" s="9"/>
       <c r="E98" s="8"/>
     </row>
-    <row r="99" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="99" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="12"/>
       <c r="B99" s="38"/>
       <c r="C99" s="39"/>
       <c r="D99" s="39"/>
@@ -1862,17 +1911,15 @@
       <c r="D103" s="9"/>
       <c r="E103" s="8"/>
     </row>
-    <row r="104" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="8"/>
       <c r="B104" s="42"/>
       <c r="C104" s="8"/>
       <c r="D104" s="9"/>
       <c r="E104" s="8"/>
     </row>
-    <row r="105" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="105" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="12"/>
       <c r="B105" s="38"/>
       <c r="C105" s="39"/>
       <c r="D105" s="39"/>
@@ -1906,17 +1953,15 @@
       <c r="D109" s="9"/>
       <c r="E109" s="8"/>
     </row>
-    <row r="110" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="8"/>
       <c r="B110" s="42"/>
       <c r="C110" s="8"/>
       <c r="D110" s="9"/>
       <c r="E110" s="8"/>
     </row>
-    <row r="111" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="111" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="12"/>
       <c r="B111" s="38"/>
       <c r="C111" s="39"/>
       <c r="D111" s="39"/>
@@ -1950,17 +1995,15 @@
       <c r="D115" s="9"/>
       <c r="E115" s="8"/>
     </row>
-    <row r="116" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="8"/>
       <c r="B116" s="42"/>
       <c r="C116" s="8"/>
       <c r="D116" s="9"/>
       <c r="E116" s="8"/>
     </row>
-    <row r="117" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="117" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="12"/>
       <c r="B117" s="38"/>
       <c r="C117" s="39"/>
       <c r="D117" s="39"/>
@@ -1994,17 +2037,15 @@
       <c r="D121" s="9"/>
       <c r="E121" s="8"/>
     </row>
-    <row r="122" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="8"/>
       <c r="B122" s="42"/>
       <c r="C122" s="8"/>
       <c r="D122" s="9"/>
       <c r="E122" s="8"/>
     </row>
-    <row r="123" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="123" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="12"/>
       <c r="B123" s="38"/>
       <c r="C123" s="39"/>
       <c r="D123" s="39"/>
@@ -2038,17 +2079,15 @@
       <c r="D127" s="9"/>
       <c r="E127" s="8"/>
     </row>
-    <row r="128" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="8"/>
       <c r="B128" s="42"/>
       <c r="C128" s="8"/>
       <c r="D128" s="9"/>
       <c r="E128" s="8"/>
     </row>
-    <row r="129" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="129" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="12"/>
       <c r="B129" s="38"/>
       <c r="C129" s="39"/>
       <c r="D129" s="39"/>
@@ -2082,17 +2121,15 @@
       <c r="D133" s="9"/>
       <c r="E133" s="8"/>
     </row>
-    <row r="134" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8"/>
       <c r="B134" s="42"/>
       <c r="C134" s="8"/>
       <c r="D134" s="9"/>
       <c r="E134" s="8"/>
     </row>
-    <row r="135" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="135" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="12"/>
       <c r="B135" s="38"/>
       <c r="C135" s="39"/>
       <c r="D135" s="39"/>
@@ -2126,17 +2163,15 @@
       <c r="D139" s="9"/>
       <c r="E139" s="8"/>
     </row>
-    <row r="140" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="8"/>
       <c r="B140" s="42"/>
       <c r="C140" s="8"/>
       <c r="D140" s="9"/>
       <c r="E140" s="8"/>
     </row>
-    <row r="141" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="141" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="12"/>
       <c r="B141" s="38"/>
       <c r="C141" s="39"/>
       <c r="D141" s="39"/>
@@ -2170,17 +2205,15 @@
       <c r="D145" s="9"/>
       <c r="E145" s="8"/>
     </row>
-    <row r="146" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="8"/>
       <c r="B146" s="42"/>
       <c r="C146" s="8"/>
       <c r="D146" s="9"/>
       <c r="E146" s="8"/>
     </row>
-    <row r="147" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="12" t="s">
-        <v>15</v>
-      </c>
+    <row r="147" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="12"/>
       <c r="B147" s="38"/>
       <c r="C147" s="39"/>
       <c r="D147" s="39"/>
@@ -2214,21 +2247,21 @@
       <c r="D151" s="9"/>
       <c r="E151" s="8"/>
     </row>
-    <row r="152" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="8"/>
       <c r="B152" s="42"/>
       <c r="C152" s="8"/>
       <c r="D152" s="9"/>
       <c r="E152" s="8"/>
     </row>
-    <row r="153" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="26" t="s">
         <v>16</v>
       </c>
       <c r="B153" s="27"/>
       <c r="C153" s="15">
         <f>MROUND(SUM(C6:C152) /60,0.2)</f>
-        <v>13.600000000000001</v>
+        <v>17.400000000000002</v>
       </c>
       <c r="D153" s="16"/>
       <c r="E153" s="17"/>
@@ -2295,7 +2328,7 @@
     <mergeCell ref="B33:E33"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C52:C56 C46:C50 C34:C38 C40:C44 C16:C20 B6 C22:C26 C28:C32 C58:C62 C148:C152 C6:C8 C76:C80 C82:C86 C70:C74 C64:C67 C88:C92 C94:C98 C100:C104 C106:C110 C112:C116 C118:C122 C124:C128 C130:C134 C136:C140 C142:C146 C10:C14" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C52:C56 C46:C50 C40:C44 C16:C20 B6 C22:C26 C28:C32 C58:C62 C148:C152 C6:C8 C76:C80 C82:C86 C70:C74 C64:C67 C88:C92 C94:C98 C100:C104 C106:C110 C112:C116 C118:C122 C124:C128 C130:C134 C136:C140 C142:C146 C10:C14 C34:C38" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B58:B62 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B46:B50 B52:B56 B64:B68 B70:B74 B76:B80 B82:B86 B88:B92 B94:B98 B100:B104 B106:B110 B112:B116 B118:B122 B124:B128 B130:B134 B136:B140 B142:B146 B148:B152 B28:B32" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
@@ -2309,7 +2342,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="30" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>

</xml_diff>

<commit_message>
chore(jdt) : maj du 10.10.26
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD8CC72-867B-4EAE-9A54-2BABF2ADE9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27A89A3E-E958-449A-91E6-0051A8651D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="73">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -254,6 +254,21 @@
   </si>
   <si>
     <t>Je fais des commentaires dans presque tout les fichiers, ajoute des rndHelpers et commente.</t>
+  </si>
+  <si>
+    <t>Nettoyage</t>
+  </si>
+  <si>
+    <t>J'améliore la propreté du code en ajoutant des commentaires et en corrigeant des petites erreurs</t>
+  </si>
+  <si>
+    <t>Je refais toute la méchanique de mouvement afin que les ennemis bougent sur des axes prédéfinis.</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Pendant que j'avance sur Ennemi, je crée un Helper "ClosestValue" et fais des tests dessus, je change par la même occasion le nom du namespace.</t>
   </si>
 </sst>
 </file>
@@ -598,22 +613,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -622,25 +645,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -975,10 +990,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="31"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -990,10 +1005,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="31"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1005,10 +1020,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="31"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1020,12 +1035,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="34"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1048,7 +1063,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="35">
+      <c r="B6" s="31">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1065,7 +1080,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="36"/>
+      <c r="B7" s="37"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1078,7 +1093,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="36"/>
+      <c r="B8" s="37"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1091,16 +1106,16 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="38"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="36"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="35">
+      <c r="B10" s="31">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1115,7 +1130,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="36"/>
+      <c r="B11" s="37"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1128,7 +1143,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="36"/>
+      <c r="B12" s="37"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1141,7 +1156,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="36"/>
+      <c r="B13" s="37"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1154,7 +1169,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="37"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1169,16 +1184,16 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="38"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="36"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="35">
+      <c r="B16" s="31">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1195,7 +1210,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="36"/>
+      <c r="B17" s="37"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1208,7 +1223,7 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="36"/>
+      <c r="B18" s="37"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
@@ -1223,7 +1238,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="36"/>
+      <c r="B19" s="37"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1236,7 +1251,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="37"/>
+      <c r="B20" s="38"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1249,16 +1264,16 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="40"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="36"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>320</v>
       </c>
-      <c r="B22" s="35">
+      <c r="B22" s="31">
         <v>46297</v>
       </c>
       <c r="C22" s="5">
@@ -1273,7 +1288,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="36"/>
+      <c r="B23" s="37"/>
       <c r="C23" s="8">
         <v>15</v>
       </c>
@@ -1286,7 +1301,7 @@
       <c r="A24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="36"/>
+      <c r="B24" s="37"/>
       <c r="C24" s="8">
         <v>160</v>
       </c>
@@ -1297,14 +1312,14 @@
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="36"/>
+      <c r="B25" s="37"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="37"/>
+      <c r="B26" s="38"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1313,16 +1328,16 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="40"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="36"/>
     </row>
     <row r="28" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="35">
+      <c r="B28" s="31">
         <v>46299</v>
       </c>
       <c r="C28" s="13">
@@ -1337,7 +1352,7 @@
       <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="36"/>
+      <c r="B29" s="37"/>
       <c r="C29" s="8">
         <v>70</v>
       </c>
@@ -1350,7 +1365,7 @@
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="36"/>
+      <c r="B30" s="37"/>
       <c r="C30" s="8">
         <v>10</v>
       </c>
@@ -1361,14 +1376,14 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="36"/>
+      <c r="B31" s="37"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="37"/>
+      <c r="B32" s="38"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1377,16 +1392,16 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="40"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="35"/>
+      <c r="D33" s="35"/>
+      <c r="E33" s="36"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="35">
+      <c r="B34" s="31">
         <v>46304</v>
       </c>
       <c r="C34" s="5">
@@ -1401,7 +1416,7 @@
       <c r="A35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="36"/>
+      <c r="B35" s="37"/>
       <c r="C35" s="5">
         <v>160</v>
       </c>
@@ -1414,7 +1429,7 @@
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="36"/>
+      <c r="B36" s="37"/>
       <c r="C36" s="8">
         <v>5</v>
       </c>
@@ -1427,7 +1442,7 @@
       <c r="A37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="36"/>
+      <c r="B37" s="37"/>
       <c r="C37" s="8">
         <v>15</v>
       </c>
@@ -1440,7 +1455,7 @@
       <c r="A38" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="37"/>
+      <c r="B38" s="38"/>
       <c r="C38" s="10">
         <v>20</v>
       </c>
@@ -1453,42 +1468,62 @@
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="38"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="39"/>
-      <c r="E39" s="40"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="35"/>
+      <c r="D39" s="35"/>
+      <c r="E39" s="36"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="4"/>
-      <c r="B40" s="35"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="25"/>
+      <c r="A40" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="31">
+        <v>46305</v>
+      </c>
+      <c r="C40" s="5">
+        <v>50</v>
+      </c>
+      <c r="D40" s="25" t="s">
+        <v>69</v>
+      </c>
       <c r="E40" s="5"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="7"/>
-      <c r="B41" s="36"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
+      <c r="A41" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B41" s="37"/>
+      <c r="C41" s="8">
+        <v>40</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="E41" s="28"/>
     </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7"/>
-      <c r="B42" s="36"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
+    <row r="42" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B42" s="37"/>
+      <c r="C42" s="8">
+        <v>20</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="E42" s="28"/>
     </row>
     <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="36"/>
+      <c r="B43" s="37"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="37"/>
+      <c r="B44" s="38"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
@@ -1497,42 +1532,42 @@
       <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="38"/>
-      <c r="C45" s="39"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="40"/>
+      <c r="B45" s="34"/>
+      <c r="C45" s="35"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
-      <c r="B46" s="35"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="5"/>
       <c r="D46" s="6"/>
       <c r="E46" s="28"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
-      <c r="B47" s="36"/>
+      <c r="B47" s="37"/>
       <c r="C47" s="8"/>
       <c r="D47" s="9"/>
       <c r="E47" s="28"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="36"/>
+      <c r="B48" s="37"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="36"/>
+      <c r="B49" s="37"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="10"/>
-      <c r="B50" s="37"/>
+      <c r="B50" s="38"/>
       <c r="C50" s="10"/>
       <c r="D50" s="11"/>
       <c r="E50" s="10"/>
@@ -1541,42 +1576,42 @@
       <c r="A51" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="38"/>
-      <c r="C51" s="39"/>
-      <c r="D51" s="39"/>
-      <c r="E51" s="40"/>
+      <c r="B51" s="34"/>
+      <c r="C51" s="35"/>
+      <c r="D51" s="35"/>
+      <c r="E51" s="36"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
-      <c r="B52" s="35"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="5"/>
       <c r="D52" s="6"/>
       <c r="E52" s="28"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7"/>
-      <c r="B53" s="36"/>
+      <c r="B53" s="37"/>
       <c r="C53" s="8"/>
       <c r="D53" s="9"/>
       <c r="E53" s="28"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="36"/>
+      <c r="B54" s="37"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="36"/>
+      <c r="B55" s="37"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="10"/>
-      <c r="B56" s="37"/>
+      <c r="B56" s="38"/>
       <c r="C56" s="10"/>
       <c r="D56" s="11"/>
       <c r="E56" s="10"/>
@@ -1585,42 +1620,42 @@
       <c r="A57" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B57" s="38"/>
-      <c r="C57" s="39"/>
-      <c r="D57" s="39"/>
-      <c r="E57" s="40"/>
+      <c r="B57" s="34"/>
+      <c r="C57" s="35"/>
+      <c r="D57" s="35"/>
+      <c r="E57" s="36"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="13"/>
-      <c r="B58" s="35"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="13"/>
       <c r="D58" s="14"/>
       <c r="E58" s="28"/>
     </row>
     <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8"/>
-      <c r="B59" s="36"/>
+      <c r="B59" s="37"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="28"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8"/>
-      <c r="B60" s="36"/>
+      <c r="B60" s="37"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8"/>
-      <c r="B61" s="36"/>
+      <c r="B61" s="37"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="8"/>
-      <c r="B62" s="37"/>
+      <c r="B62" s="38"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
@@ -1629,627 +1664,627 @@
       <c r="A63" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B63" s="38"/>
-      <c r="C63" s="39"/>
-      <c r="D63" s="39"/>
-      <c r="E63" s="40"/>
+      <c r="B63" s="34"/>
+      <c r="C63" s="35"/>
+      <c r="D63" s="35"/>
+      <c r="E63" s="36"/>
     </row>
     <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8"/>
-      <c r="B64" s="35"/>
+      <c r="B64" s="31"/>
       <c r="C64" s="13"/>
       <c r="D64" s="14"/>
       <c r="E64" s="28"/>
     </row>
     <row r="65" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="36"/>
+      <c r="B65" s="37"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8"/>
-      <c r="B66" s="36"/>
+      <c r="B66" s="37"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8"/>
-      <c r="B67" s="36"/>
+      <c r="B67" s="37"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="8"/>
-      <c r="B68" s="37"/>
+      <c r="B68" s="38"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="12"/>
-      <c r="B69" s="38"/>
-      <c r="C69" s="39"/>
-      <c r="D69" s="39"/>
-      <c r="E69" s="40"/>
+      <c r="B69" s="34"/>
+      <c r="C69" s="35"/>
+      <c r="D69" s="35"/>
+      <c r="E69" s="36"/>
     </row>
     <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8"/>
-      <c r="B70" s="35"/>
+      <c r="B70" s="31"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="28"/>
     </row>
     <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8"/>
-      <c r="B71" s="36"/>
+      <c r="B71" s="37"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="36"/>
+      <c r="B72" s="37"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="8"/>
-      <c r="B73" s="36"/>
+      <c r="B73" s="37"/>
       <c r="C73" s="8"/>
       <c r="D73" s="9"/>
       <c r="E73" s="8"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="8"/>
-      <c r="B74" s="37"/>
+      <c r="B74" s="38"/>
       <c r="C74" s="8"/>
       <c r="D74" s="9"/>
       <c r="E74" s="8"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="12"/>
-      <c r="B75" s="38"/>
-      <c r="C75" s="39"/>
-      <c r="D75" s="39"/>
-      <c r="E75" s="40"/>
+      <c r="B75" s="34"/>
+      <c r="C75" s="35"/>
+      <c r="D75" s="35"/>
+      <c r="E75" s="36"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="13"/>
-      <c r="B76" s="35"/>
+      <c r="B76" s="31"/>
       <c r="C76" s="13"/>
       <c r="D76" s="14"/>
       <c r="E76" s="28"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="8"/>
-      <c r="B77" s="36"/>
+      <c r="B77" s="37"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="8"/>
-      <c r="B78" s="36"/>
+      <c r="B78" s="37"/>
       <c r="C78" s="8"/>
       <c r="D78" s="29"/>
       <c r="E78" s="8"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="8"/>
-      <c r="B79" s="36"/>
+      <c r="B79" s="37"/>
       <c r="C79" s="8"/>
       <c r="D79" s="9"/>
       <c r="E79" s="8"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="8"/>
-      <c r="B80" s="37"/>
+      <c r="B80" s="38"/>
       <c r="C80" s="8"/>
       <c r="D80" s="9"/>
       <c r="E80" s="8"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="12"/>
-      <c r="B81" s="38"/>
-      <c r="C81" s="39"/>
-      <c r="D81" s="39"/>
-      <c r="E81" s="40"/>
+      <c r="B81" s="34"/>
+      <c r="C81" s="35"/>
+      <c r="D81" s="35"/>
+      <c r="E81" s="36"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="13"/>
-      <c r="B82" s="35"/>
+      <c r="B82" s="31"/>
       <c r="C82" s="13"/>
       <c r="D82" s="14"/>
       <c r="E82" s="28"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="13"/>
-      <c r="B83" s="41"/>
+      <c r="B83" s="32"/>
       <c r="C83" s="8"/>
       <c r="D83" s="14"/>
       <c r="E83" s="28"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="8"/>
-      <c r="B84" s="41"/>
+      <c r="B84" s="32"/>
       <c r="C84" s="8"/>
       <c r="D84" s="9"/>
       <c r="E84" s="8"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="8"/>
-      <c r="B85" s="41"/>
+      <c r="B85" s="32"/>
       <c r="C85" s="8"/>
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
     <row r="86" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="8"/>
-      <c r="B86" s="42"/>
+      <c r="B86" s="33"/>
       <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="12"/>
-      <c r="B87" s="38"/>
-      <c r="C87" s="39"/>
-      <c r="D87" s="39"/>
-      <c r="E87" s="40"/>
+      <c r="B87" s="34"/>
+      <c r="C87" s="35"/>
+      <c r="D87" s="35"/>
+      <c r="E87" s="36"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="13"/>
-      <c r="B88" s="35"/>
+      <c r="B88" s="31"/>
       <c r="C88" s="13"/>
       <c r="D88" s="14"/>
       <c r="E88" s="28"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="13"/>
-      <c r="B89" s="41"/>
+      <c r="B89" s="32"/>
       <c r="C89" s="8"/>
       <c r="D89" s="14"/>
       <c r="E89" s="28"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="8"/>
-      <c r="B90" s="41"/>
+      <c r="B90" s="32"/>
       <c r="C90" s="8"/>
       <c r="D90" s="9"/>
       <c r="E90" s="8"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="8"/>
-      <c r="B91" s="41"/>
+      <c r="B91" s="32"/>
       <c r="C91" s="8"/>
       <c r="D91" s="9"/>
       <c r="E91" s="8"/>
     </row>
     <row r="92" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="8"/>
-      <c r="B92" s="42"/>
+      <c r="B92" s="33"/>
       <c r="C92" s="8"/>
       <c r="D92" s="9"/>
       <c r="E92" s="8"/>
     </row>
     <row r="93" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="12"/>
-      <c r="B93" s="38"/>
-      <c r="C93" s="39"/>
-      <c r="D93" s="39"/>
-      <c r="E93" s="40"/>
+      <c r="B93" s="34"/>
+      <c r="C93" s="35"/>
+      <c r="D93" s="35"/>
+      <c r="E93" s="36"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="13"/>
-      <c r="B94" s="35"/>
+      <c r="B94" s="31"/>
       <c r="C94" s="13"/>
       <c r="D94" s="14"/>
       <c r="E94" s="28"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="13"/>
-      <c r="B95" s="41"/>
+      <c r="B95" s="32"/>
       <c r="C95" s="8"/>
       <c r="D95" s="14"/>
       <c r="E95" s="28"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="8"/>
-      <c r="B96" s="41"/>
+      <c r="B96" s="32"/>
       <c r="C96" s="8"/>
       <c r="D96" s="9"/>
       <c r="E96" s="8"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="8"/>
-      <c r="B97" s="41"/>
+      <c r="B97" s="32"/>
       <c r="C97" s="8"/>
       <c r="D97" s="9"/>
       <c r="E97" s="8"/>
     </row>
     <row r="98" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="8"/>
-      <c r="B98" s="42"/>
+      <c r="B98" s="33"/>
       <c r="C98" s="8"/>
       <c r="D98" s="9"/>
       <c r="E98" s="8"/>
     </row>
     <row r="99" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="12"/>
-      <c r="B99" s="38"/>
-      <c r="C99" s="39"/>
-      <c r="D99" s="39"/>
-      <c r="E99" s="40"/>
+      <c r="B99" s="34"/>
+      <c r="C99" s="35"/>
+      <c r="D99" s="35"/>
+      <c r="E99" s="36"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="13"/>
-      <c r="B100" s="35"/>
+      <c r="B100" s="31"/>
       <c r="C100" s="13"/>
       <c r="D100" s="14"/>
       <c r="E100" s="28"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="13"/>
-      <c r="B101" s="41"/>
+      <c r="B101" s="32"/>
       <c r="C101" s="8"/>
       <c r="D101" s="14"/>
       <c r="E101" s="28"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="8"/>
-      <c r="B102" s="41"/>
+      <c r="B102" s="32"/>
       <c r="C102" s="8"/>
       <c r="D102" s="9"/>
       <c r="E102" s="8"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="8"/>
-      <c r="B103" s="41"/>
+      <c r="B103" s="32"/>
       <c r="C103" s="8"/>
       <c r="D103" s="9"/>
       <c r="E103" s="8"/>
     </row>
     <row r="104" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="8"/>
-      <c r="B104" s="42"/>
+      <c r="B104" s="33"/>
       <c r="C104" s="8"/>
       <c r="D104" s="9"/>
       <c r="E104" s="8"/>
     </row>
     <row r="105" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="12"/>
-      <c r="B105" s="38"/>
-      <c r="C105" s="39"/>
-      <c r="D105" s="39"/>
-      <c r="E105" s="40"/>
+      <c r="B105" s="34"/>
+      <c r="C105" s="35"/>
+      <c r="D105" s="35"/>
+      <c r="E105" s="36"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="13"/>
-      <c r="B106" s="35"/>
+      <c r="B106" s="31"/>
       <c r="C106" s="13"/>
       <c r="D106" s="14"/>
       <c r="E106" s="28"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="13"/>
-      <c r="B107" s="41"/>
+      <c r="B107" s="32"/>
       <c r="C107" s="8"/>
       <c r="D107" s="14"/>
       <c r="E107" s="28"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="8"/>
-      <c r="B108" s="41"/>
+      <c r="B108" s="32"/>
       <c r="C108" s="8"/>
       <c r="D108" s="9"/>
       <c r="E108" s="8"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="8"/>
-      <c r="B109" s="41"/>
+      <c r="B109" s="32"/>
       <c r="C109" s="8"/>
       <c r="D109" s="9"/>
       <c r="E109" s="8"/>
     </row>
     <row r="110" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="8"/>
-      <c r="B110" s="42"/>
+      <c r="B110" s="33"/>
       <c r="C110" s="8"/>
       <c r="D110" s="9"/>
       <c r="E110" s="8"/>
     </row>
     <row r="111" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="12"/>
-      <c r="B111" s="38"/>
-      <c r="C111" s="39"/>
-      <c r="D111" s="39"/>
-      <c r="E111" s="40"/>
+      <c r="B111" s="34"/>
+      <c r="C111" s="35"/>
+      <c r="D111" s="35"/>
+      <c r="E111" s="36"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="13"/>
-      <c r="B112" s="35"/>
+      <c r="B112" s="31"/>
       <c r="C112" s="13"/>
       <c r="D112" s="14"/>
       <c r="E112" s="28"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="13"/>
-      <c r="B113" s="41"/>
+      <c r="B113" s="32"/>
       <c r="C113" s="8"/>
       <c r="D113" s="14"/>
       <c r="E113" s="28"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="8"/>
-      <c r="B114" s="41"/>
+      <c r="B114" s="32"/>
       <c r="C114" s="8"/>
       <c r="D114" s="9"/>
       <c r="E114" s="8"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="8"/>
-      <c r="B115" s="41"/>
+      <c r="B115" s="32"/>
       <c r="C115" s="8"/>
       <c r="D115" s="9"/>
       <c r="E115" s="8"/>
     </row>
     <row r="116" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="8"/>
-      <c r="B116" s="42"/>
+      <c r="B116" s="33"/>
       <c r="C116" s="8"/>
       <c r="D116" s="9"/>
       <c r="E116" s="8"/>
     </row>
     <row r="117" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="12"/>
-      <c r="B117" s="38"/>
-      <c r="C117" s="39"/>
-      <c r="D117" s="39"/>
-      <c r="E117" s="40"/>
+      <c r="B117" s="34"/>
+      <c r="C117" s="35"/>
+      <c r="D117" s="35"/>
+      <c r="E117" s="36"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="13"/>
-      <c r="B118" s="35"/>
+      <c r="B118" s="31"/>
       <c r="C118" s="13"/>
       <c r="D118" s="14"/>
       <c r="E118" s="28"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="13"/>
-      <c r="B119" s="41"/>
+      <c r="B119" s="32"/>
       <c r="C119" s="8"/>
       <c r="D119" s="14"/>
       <c r="E119" s="28"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="8"/>
-      <c r="B120" s="41"/>
+      <c r="B120" s="32"/>
       <c r="C120" s="8"/>
       <c r="D120" s="9"/>
       <c r="E120" s="8"/>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="8"/>
-      <c r="B121" s="41"/>
+      <c r="B121" s="32"/>
       <c r="C121" s="8"/>
       <c r="D121" s="9"/>
       <c r="E121" s="8"/>
     </row>
     <row r="122" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="8"/>
-      <c r="B122" s="42"/>
+      <c r="B122" s="33"/>
       <c r="C122" s="8"/>
       <c r="D122" s="9"/>
       <c r="E122" s="8"/>
     </row>
     <row r="123" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="12"/>
-      <c r="B123" s="38"/>
-      <c r="C123" s="39"/>
-      <c r="D123" s="39"/>
-      <c r="E123" s="40"/>
+      <c r="B123" s="34"/>
+      <c r="C123" s="35"/>
+      <c r="D123" s="35"/>
+      <c r="E123" s="36"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="13"/>
-      <c r="B124" s="35"/>
+      <c r="B124" s="31"/>
       <c r="C124" s="13"/>
       <c r="D124" s="14"/>
       <c r="E124" s="28"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="13"/>
-      <c r="B125" s="41"/>
+      <c r="B125" s="32"/>
       <c r="C125" s="8"/>
       <c r="D125" s="14"/>
       <c r="E125" s="28"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="8"/>
-      <c r="B126" s="41"/>
+      <c r="B126" s="32"/>
       <c r="C126" s="8"/>
       <c r="D126" s="9"/>
       <c r="E126" s="8"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="8"/>
-      <c r="B127" s="41"/>
+      <c r="B127" s="32"/>
       <c r="C127" s="8"/>
       <c r="D127" s="9"/>
       <c r="E127" s="8"/>
     </row>
     <row r="128" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="8"/>
-      <c r="B128" s="42"/>
+      <c r="B128" s="33"/>
       <c r="C128" s="8"/>
       <c r="D128" s="9"/>
       <c r="E128" s="8"/>
     </row>
     <row r="129" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="12"/>
-      <c r="B129" s="38"/>
-      <c r="C129" s="39"/>
-      <c r="D129" s="39"/>
-      <c r="E129" s="40"/>
+      <c r="B129" s="34"/>
+      <c r="C129" s="35"/>
+      <c r="D129" s="35"/>
+      <c r="E129" s="36"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="13"/>
-      <c r="B130" s="35"/>
+      <c r="B130" s="31"/>
       <c r="C130" s="13"/>
       <c r="D130" s="14"/>
       <c r="E130" s="28"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="13"/>
-      <c r="B131" s="41"/>
+      <c r="B131" s="32"/>
       <c r="C131" s="8"/>
       <c r="D131" s="14"/>
       <c r="E131" s="28"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="8"/>
-      <c r="B132" s="41"/>
+      <c r="B132" s="32"/>
       <c r="C132" s="8"/>
       <c r="D132" s="9"/>
       <c r="E132" s="8"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="8"/>
-      <c r="B133" s="41"/>
+      <c r="B133" s="32"/>
       <c r="C133" s="8"/>
       <c r="D133" s="9"/>
       <c r="E133" s="8"/>
     </row>
     <row r="134" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8"/>
-      <c r="B134" s="42"/>
+      <c r="B134" s="33"/>
       <c r="C134" s="8"/>
       <c r="D134" s="9"/>
       <c r="E134" s="8"/>
     </row>
     <row r="135" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="12"/>
-      <c r="B135" s="38"/>
-      <c r="C135" s="39"/>
-      <c r="D135" s="39"/>
-      <c r="E135" s="40"/>
+      <c r="B135" s="34"/>
+      <c r="C135" s="35"/>
+      <c r="D135" s="35"/>
+      <c r="E135" s="36"/>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="13"/>
-      <c r="B136" s="35"/>
+      <c r="B136" s="31"/>
       <c r="C136" s="13"/>
       <c r="D136" s="14"/>
       <c r="E136" s="28"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="13"/>
-      <c r="B137" s="41"/>
+      <c r="B137" s="32"/>
       <c r="C137" s="8"/>
       <c r="D137" s="14"/>
       <c r="E137" s="28"/>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="8"/>
-      <c r="B138" s="41"/>
+      <c r="B138" s="32"/>
       <c r="C138" s="8"/>
       <c r="D138" s="9"/>
       <c r="E138" s="8"/>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="8"/>
-      <c r="B139" s="41"/>
+      <c r="B139" s="32"/>
       <c r="C139" s="8"/>
       <c r="D139" s="9"/>
       <c r="E139" s="8"/>
     </row>
     <row r="140" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="8"/>
-      <c r="B140" s="42"/>
+      <c r="B140" s="33"/>
       <c r="C140" s="8"/>
       <c r="D140" s="9"/>
       <c r="E140" s="8"/>
     </row>
     <row r="141" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="12"/>
-      <c r="B141" s="38"/>
-      <c r="C141" s="39"/>
-      <c r="D141" s="39"/>
-      <c r="E141" s="40"/>
+      <c r="B141" s="34"/>
+      <c r="C141" s="35"/>
+      <c r="D141" s="35"/>
+      <c r="E141" s="36"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="13"/>
-      <c r="B142" s="35"/>
+      <c r="B142" s="31"/>
       <c r="C142" s="13"/>
       <c r="D142" s="14"/>
       <c r="E142" s="28"/>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="13"/>
-      <c r="B143" s="41"/>
+      <c r="B143" s="32"/>
       <c r="C143" s="8"/>
       <c r="D143" s="14"/>
       <c r="E143" s="28"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="8"/>
-      <c r="B144" s="41"/>
+      <c r="B144" s="32"/>
       <c r="C144" s="8"/>
       <c r="D144" s="9"/>
       <c r="E144" s="8"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="8"/>
-      <c r="B145" s="41"/>
+      <c r="B145" s="32"/>
       <c r="C145" s="8"/>
       <c r="D145" s="9"/>
       <c r="E145" s="8"/>
     </row>
     <row r="146" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="8"/>
-      <c r="B146" s="42"/>
+      <c r="B146" s="33"/>
       <c r="C146" s="8"/>
       <c r="D146" s="9"/>
       <c r="E146" s="8"/>
     </row>
     <row r="147" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="12"/>
-      <c r="B147" s="38"/>
-      <c r="C147" s="39"/>
-      <c r="D147" s="39"/>
-      <c r="E147" s="40"/>
+      <c r="B147" s="34"/>
+      <c r="C147" s="35"/>
+      <c r="D147" s="35"/>
+      <c r="E147" s="36"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="13"/>
-      <c r="B148" s="35"/>
+      <c r="B148" s="31"/>
       <c r="C148" s="13"/>
       <c r="D148" s="14"/>
       <c r="E148" s="28"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="13"/>
-      <c r="B149" s="41"/>
+      <c r="B149" s="32"/>
       <c r="C149" s="8"/>
       <c r="D149" s="14"/>
       <c r="E149" s="28"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="8"/>
-      <c r="B150" s="41"/>
+      <c r="B150" s="32"/>
       <c r="C150" s="8"/>
       <c r="D150" s="9"/>
       <c r="E150" s="8"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="8"/>
-      <c r="B151" s="41"/>
+      <c r="B151" s="32"/>
       <c r="C151" s="8"/>
       <c r="D151" s="9"/>
       <c r="E151" s="8"/>
     </row>
     <row r="152" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="8"/>
-      <c r="B152" s="42"/>
+      <c r="B152" s="33"/>
       <c r="C152" s="8"/>
       <c r="D152" s="9"/>
       <c r="E152" s="8"/>
@@ -2261,7 +2296,7 @@
       <c r="B153" s="27"/>
       <c r="C153" s="15">
         <f>MROUND(SUM(C6:C152) /60,0.2)</f>
-        <v>17.400000000000002</v>
+        <v>19.200000000000003</v>
       </c>
       <c r="D153" s="16"/>
       <c r="E153" s="17"/>
@@ -2273,43 +2308,6 @@
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B142:B146"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:B152"/>
-    <mergeCell ref="B129:E129"/>
-    <mergeCell ref="B130:B134"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B136:B140"/>
-    <mergeCell ref="B141:E141"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B118:B122"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B124:B128"/>
-    <mergeCell ref="B100:B104"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="B106:B110"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B94:B98"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:B50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="B76:B80"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -2326,6 +2324,43 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:B50"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B52:B56"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B88:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B94:B98"/>
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B100:B104"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="B106:B110"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B112:B116"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B118:B122"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B124:B128"/>
+    <mergeCell ref="B142:B146"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:B152"/>
+    <mergeCell ref="B129:E129"/>
+    <mergeCell ref="B130:B134"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B136:B140"/>
+    <mergeCell ref="B141:E141"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C52:C56 C46:C50 C40:C44 C16:C20 B6 C22:C26 C28:C32 C58:C62 C148:C152 C6:C8 C76:C80 C82:C86 C70:C74 C64:C67 C88:C92 C94:C98 C100:C104 C106:C110 C112:C116 C118:C122 C124:C128 C130:C134 C136:C140 C142:C146 C10:C14 C34:C38" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -2342,7 +2377,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="29" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="28" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2360,15 +2395,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -2550,6 +2576,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -2567,14 +2602,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2590,4 +2617,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : maj du 11.10.26
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27A89A3E-E958-449A-91E6-0051A8651D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACCA033-32E7-4434-A191-59E17881673B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$153</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$61</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="87">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -269,6 +269,48 @@
   </si>
   <si>
     <t>Pendant que j'avance sur Ennemi, je crée un Helper "ClosestValue" et fais des tests dessus, je change par la même occasion le nom du namespace.</t>
+  </si>
+  <si>
+    <t>Objectifs</t>
+  </si>
+  <si>
+    <t>Je crée une methode qui définis les objectifs à partir des axes dynamiquement et fais des tests dessus qui m'aident à la réparer.</t>
+  </si>
+  <si>
+    <t>axes</t>
+  </si>
+  <si>
+    <t>J'adapte tout le système d'axes des ennemis pour qu'il ne dépende que des axes définis au début, les objectifs ont une direction au lieu de simplement empêcher de sortir des axes.</t>
+  </si>
+  <si>
+    <t>spawners</t>
+  </si>
+  <si>
+    <t>J'adapte les spawners pour qu'ils soient aussi en haut de l'écran et qu'ils soient assignés automatiquement</t>
+  </si>
+  <si>
+    <t>J'essaye d'empêcher que les ennemis choisissent un objectif en diagonale et autres problèmes de mouvements liés.</t>
+  </si>
+  <si>
+    <t>Je corrige un peu les US en mettant "je veux" au lieu de "j'aimerais" et en changeant les images.</t>
+  </si>
+  <si>
+    <t>Vie joueur</t>
+  </si>
+  <si>
+    <t>J'ajoute rapidement la vie du joueur.</t>
+  </si>
+  <si>
+    <t>Dégats joueur</t>
+  </si>
+  <si>
+    <t>J'ajoute les dégats du joueur (Les ennemis réapparaissent bizarrement pour le moment).</t>
+  </si>
+  <si>
+    <t>Rapport</t>
+  </si>
+  <si>
+    <t>Je remplis le rapport, chapitre IA, tests, bilan produit et conception.</t>
   </si>
 </sst>
 </file>
@@ -514,7 +556,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -605,10 +647,6 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -637,12 +675,36 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -973,7 +1035,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -990,10 +1052,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="39"/>
+      <c r="C1" s="44"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -1005,10 +1067,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="39"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1020,10 +1082,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="39"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1035,12 +1097,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1063,7 +1125,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="31">
+      <c r="B6" s="36">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1080,7 +1142,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="37"/>
+      <c r="B7" s="39"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1093,7 +1155,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="37"/>
+      <c r="B8" s="39"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1106,16 +1168,16 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="34"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
+      <c r="B9" s="41"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="43"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="36">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1130,7 +1192,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="37"/>
+      <c r="B11" s="39"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1143,7 +1205,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="37"/>
+      <c r="B12" s="39"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1156,7 +1218,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="37"/>
+      <c r="B13" s="39"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1169,7 +1231,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="38"/>
+      <c r="B14" s="40"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1184,16 +1246,16 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="43"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="31">
+      <c r="B16" s="36">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1210,7 +1272,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="37"/>
+      <c r="B17" s="39"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1223,14 +1285,14 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="37"/>
+      <c r="B18" s="39"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="30" t="s">
+      <c r="E18" s="29" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1238,7 +1300,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="37"/>
+      <c r="B19" s="39"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1251,7 +1313,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="38"/>
+      <c r="B20" s="40"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1264,16 +1326,16 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="36"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="43"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>320</v>
       </c>
-      <c r="B22" s="31">
+      <c r="B22" s="36">
         <v>46297</v>
       </c>
       <c r="C22" s="5">
@@ -1288,7 +1350,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="37"/>
+      <c r="B23" s="39"/>
       <c r="C23" s="8">
         <v>15</v>
       </c>
@@ -1301,7 +1363,7 @@
       <c r="A24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="37"/>
+      <c r="B24" s="39"/>
       <c r="C24" s="8">
         <v>160</v>
       </c>
@@ -1312,14 +1374,14 @@
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="37"/>
+      <c r="B25" s="39"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="38"/>
+      <c r="B26" s="40"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1328,16 +1390,16 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="34"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="36"/>
+      <c r="B27" s="41"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="43"/>
     </row>
     <row r="28" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="31">
+      <c r="B28" s="36">
         <v>46299</v>
       </c>
       <c r="C28" s="13">
@@ -1352,7 +1414,7 @@
       <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="37"/>
+      <c r="B29" s="39"/>
       <c r="C29" s="8">
         <v>70</v>
       </c>
@@ -1365,7 +1427,7 @@
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="37"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="8">
         <v>10</v>
       </c>
@@ -1376,14 +1438,14 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="37"/>
+      <c r="B31" s="39"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="38"/>
+      <c r="B32" s="40"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1392,16 +1454,16 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="36"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="43"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="31">
+      <c r="B34" s="36">
         <v>46304</v>
       </c>
       <c r="C34" s="5">
@@ -1416,7 +1478,7 @@
       <c r="A35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="37"/>
+      <c r="B35" s="39"/>
       <c r="C35" s="5">
         <v>160</v>
       </c>
@@ -1429,7 +1491,7 @@
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="37"/>
+      <c r="B36" s="39"/>
       <c r="C36" s="8">
         <v>5</v>
       </c>
@@ -1442,7 +1504,7 @@
       <c r="A37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="37"/>
+      <c r="B37" s="39"/>
       <c r="C37" s="8">
         <v>15</v>
       </c>
@@ -1455,7 +1517,7 @@
       <c r="A38" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="38"/>
+      <c r="B38" s="40"/>
       <c r="C38" s="10">
         <v>20</v>
       </c>
@@ -1468,20 +1530,20 @@
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="34"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="36"/>
+      <c r="B39" s="41"/>
+      <c r="C39" s="42"/>
+      <c r="D39" s="42"/>
+      <c r="E39" s="43"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="31">
+      <c r="B40" s="36">
         <v>46305</v>
       </c>
       <c r="C40" s="5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D40" s="25" t="s">
         <v>69</v>
@@ -1492,9 +1554,9 @@
       <c r="A41" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="37"/>
+      <c r="B41" s="39"/>
       <c r="C41" s="8">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>70</v>
@@ -1505,7 +1567,7 @@
       <c r="A42" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="37"/>
+      <c r="B42" s="39"/>
       <c r="C42" s="8">
         <v>20</v>
       </c>
@@ -1516,14 +1578,14 @@
     </row>
     <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="37"/>
+      <c r="B43" s="39"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="38"/>
+      <c r="B44" s="40"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
@@ -1532,787 +1594,277 @@
       <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="34"/>
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="36"/>
+      <c r="B45" s="41"/>
+      <c r="C45" s="42"/>
+      <c r="D45" s="42"/>
+      <c r="E45" s="43"/>
     </row>
     <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="4"/>
-      <c r="B46" s="31"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="6"/>
+      <c r="A46" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B46" s="36">
+        <v>46306</v>
+      </c>
+      <c r="C46" s="5">
+        <v>25</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="E46" s="28"/>
     </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="7"/>
+    <row r="47" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7" t="s">
+        <v>75</v>
+      </c>
       <c r="B47" s="37"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
+      <c r="C47" s="8">
+        <v>40</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>76</v>
+      </c>
       <c r="E47" s="28"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7"/>
+      <c r="A48" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="B48" s="37"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
+      <c r="C48" s="8">
+        <v>40</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="7"/>
+      <c r="A49" s="7" t="s">
+        <v>73</v>
+      </c>
       <c r="B49" s="37"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
+      <c r="C49" s="8">
+        <v>70</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>79</v>
+      </c>
       <c r="E49" s="8"/>
     </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="10"/>
-      <c r="B50" s="38"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="11"/>
+    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B50" s="37"/>
+      <c r="C50" s="10">
+        <v>15</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>80</v>
+      </c>
       <c r="E50" s="10"/>
     </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
+    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B51" s="37"/>
+      <c r="C51" s="10">
+        <v>20</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="E51" s="10"/>
+    </row>
+    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B52" s="37"/>
+      <c r="C52" s="10">
+        <v>20</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52" s="10"/>
+    </row>
+    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B53" s="37"/>
+      <c r="C53" s="10">
+        <v>30</v>
+      </c>
+      <c r="D53" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E53" s="10"/>
+    </row>
+    <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="10"/>
+      <c r="B54" s="38"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="10"/>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="34"/>
-      <c r="C51" s="35"/>
-      <c r="D51" s="35"/>
-      <c r="E51" s="36"/>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="4"/>
-      <c r="B52" s="31"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="28"/>
-    </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="28"/>
-    </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="7"/>
-      <c r="B54" s="37"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="8"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="7"/>
-      <c r="B55" s="37"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="8"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10"/>
-      <c r="B56" s="38"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="10"/>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B57" s="34"/>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="36"/>
+      <c r="B55" s="41"/>
+      <c r="C55" s="42"/>
+      <c r="D55" s="42"/>
+      <c r="E55" s="43"/>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="4"/>
+      <c r="B56" s="36"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="28"/>
+    </row>
+    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="37"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="28"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="13"/>
-      <c r="B58" s="31"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="28"/>
+      <c r="A58" s="7"/>
+      <c r="B58" s="37"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="8"/>
+      <c r="A59" s="7"/>
       <c r="B59" s="37"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
-      <c r="E59" s="28"/>
-    </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="8"/>
-      <c r="B60" s="37"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="8"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="8"/>
-      <c r="B61" s="37"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="8"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="8"/>
-      <c r="B62" s="38"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B63" s="34"/>
-      <c r="C63" s="35"/>
-      <c r="D63" s="35"/>
-      <c r="E63" s="36"/>
-    </row>
-    <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="8"/>
-      <c r="B64" s="31"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="28"/>
-    </row>
-    <row r="65" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="37"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="8"/>
-      <c r="B66" s="37"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="8"/>
-    </row>
-    <row r="67" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="8"/>
-      <c r="B67" s="37"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="8"/>
-      <c r="B68" s="38"/>
-      <c r="E68" s="8"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="12"/>
-      <c r="B69" s="34"/>
-      <c r="C69" s="35"/>
-      <c r="D69" s="35"/>
-      <c r="E69" s="36"/>
-    </row>
-    <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="8"/>
-      <c r="B70" s="31"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="28"/>
-    </row>
-    <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="8"/>
-      <c r="B71" s="37"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="8"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="8"/>
-      <c r="B72" s="37"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="8"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="8"/>
-      <c r="B73" s="37"/>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="8"/>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="8"/>
-      <c r="B74" s="38"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="9"/>
-      <c r="E74" s="8"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="12"/>
-      <c r="B75" s="34"/>
-      <c r="C75" s="35"/>
-      <c r="D75" s="35"/>
-      <c r="E75" s="36"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="13"/>
-      <c r="B76" s="31"/>
-      <c r="C76" s="13"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="28"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="8"/>
-      <c r="B77" s="37"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="8"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="8"/>
-      <c r="B78" s="37"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="29"/>
-      <c r="E78" s="8"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="8"/>
-      <c r="B79" s="37"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="8"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="8"/>
-      <c r="B80" s="38"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="9"/>
-      <c r="E80" s="8"/>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="12"/>
-      <c r="B81" s="34"/>
-      <c r="C81" s="35"/>
-      <c r="D81" s="35"/>
-      <c r="E81" s="36"/>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="13"/>
-      <c r="B82" s="31"/>
-      <c r="C82" s="13"/>
-      <c r="D82" s="14"/>
-      <c r="E82" s="28"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="13"/>
-      <c r="B83" s="32"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="14"/>
-      <c r="E83" s="28"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="8"/>
-      <c r="B84" s="32"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="9"/>
-      <c r="E84" s="8"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="8"/>
-      <c r="B85" s="32"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="9"/>
-      <c r="E85" s="8"/>
-    </row>
-    <row r="86" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="8"/>
-      <c r="B86" s="33"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="9"/>
-      <c r="E86" s="8"/>
-    </row>
-    <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="12"/>
-      <c r="B87" s="34"/>
-      <c r="C87" s="35"/>
-      <c r="D87" s="35"/>
-      <c r="E87" s="36"/>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="13"/>
-      <c r="B88" s="31"/>
-      <c r="C88" s="13"/>
-      <c r="D88" s="14"/>
-      <c r="E88" s="28"/>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="13"/>
-      <c r="B89" s="32"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="14"/>
-      <c r="E89" s="28"/>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="8"/>
-      <c r="B90" s="32"/>
-      <c r="C90" s="8"/>
-      <c r="D90" s="9"/>
-      <c r="E90" s="8"/>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="8"/>
-      <c r="B91" s="32"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="9"/>
-      <c r="E91" s="8"/>
-    </row>
-    <row r="92" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="8"/>
-      <c r="B92" s="33"/>
-      <c r="C92" s="8"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="8"/>
-    </row>
-    <row r="93" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="12"/>
-      <c r="B93" s="34"/>
-      <c r="C93" s="35"/>
-      <c r="D93" s="35"/>
-      <c r="E93" s="36"/>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="13"/>
-      <c r="B94" s="31"/>
-      <c r="C94" s="13"/>
-      <c r="D94" s="14"/>
-      <c r="E94" s="28"/>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="13"/>
-      <c r="B95" s="32"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="14"/>
-      <c r="E95" s="28"/>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="8"/>
-      <c r="B96" s="32"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="9"/>
-      <c r="E96" s="8"/>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="8"/>
-      <c r="B97" s="32"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="9"/>
-      <c r="E97" s="8"/>
-    </row>
-    <row r="98" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="8"/>
-      <c r="B98" s="33"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="9"/>
-      <c r="E98" s="8"/>
-    </row>
-    <row r="99" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="12"/>
-      <c r="B99" s="34"/>
-      <c r="C99" s="35"/>
-      <c r="D99" s="35"/>
-      <c r="E99" s="36"/>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="13"/>
-      <c r="B100" s="31"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="14"/>
-      <c r="E100" s="28"/>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="13"/>
-      <c r="B101" s="32"/>
-      <c r="C101" s="8"/>
-      <c r="D101" s="14"/>
-      <c r="E101" s="28"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="8"/>
-      <c r="B102" s="32"/>
-      <c r="C102" s="8"/>
-      <c r="D102" s="9"/>
-      <c r="E102" s="8"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="8"/>
-      <c r="B103" s="32"/>
-      <c r="C103" s="8"/>
-      <c r="D103" s="9"/>
-      <c r="E103" s="8"/>
-    </row>
-    <row r="104" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A104" s="8"/>
-      <c r="B104" s="33"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="9"/>
-      <c r="E104" s="8"/>
-    </row>
-    <row r="105" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="12"/>
-      <c r="B105" s="34"/>
-      <c r="C105" s="35"/>
-      <c r="D105" s="35"/>
-      <c r="E105" s="36"/>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="13"/>
-      <c r="B106" s="31"/>
-      <c r="C106" s="13"/>
-      <c r="D106" s="14"/>
-      <c r="E106" s="28"/>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="13"/>
-      <c r="B107" s="32"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="14"/>
-      <c r="E107" s="28"/>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="8"/>
-      <c r="B108" s="32"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="9"/>
-      <c r="E108" s="8"/>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="8"/>
-      <c r="B109" s="32"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="9"/>
-      <c r="E109" s="8"/>
-    </row>
-    <row r="110" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="8"/>
-      <c r="B110" s="33"/>
-      <c r="C110" s="8"/>
-      <c r="D110" s="9"/>
-      <c r="E110" s="8"/>
-    </row>
-    <row r="111" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="12"/>
-      <c r="B111" s="34"/>
-      <c r="C111" s="35"/>
-      <c r="D111" s="35"/>
-      <c r="E111" s="36"/>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="13"/>
-      <c r="B112" s="31"/>
-      <c r="C112" s="13"/>
-      <c r="D112" s="14"/>
-      <c r="E112" s="28"/>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="13"/>
-      <c r="B113" s="32"/>
-      <c r="C113" s="8"/>
-      <c r="D113" s="14"/>
-      <c r="E113" s="28"/>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="8"/>
-      <c r="B114" s="32"/>
-      <c r="C114" s="8"/>
-      <c r="D114" s="9"/>
-      <c r="E114" s="8"/>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="8"/>
-      <c r="B115" s="32"/>
-      <c r="C115" s="8"/>
-      <c r="D115" s="9"/>
-      <c r="E115" s="8"/>
-    </row>
-    <row r="116" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="8"/>
-      <c r="B116" s="33"/>
-      <c r="C116" s="8"/>
-      <c r="D116" s="9"/>
-      <c r="E116" s="8"/>
-    </row>
-    <row r="117" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="12"/>
-      <c r="B117" s="34"/>
-      <c r="C117" s="35"/>
-      <c r="D117" s="35"/>
-      <c r="E117" s="36"/>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" s="13"/>
-      <c r="B118" s="31"/>
-      <c r="C118" s="13"/>
-      <c r="D118" s="14"/>
-      <c r="E118" s="28"/>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="13"/>
-      <c r="B119" s="32"/>
-      <c r="C119" s="8"/>
-      <c r="D119" s="14"/>
-      <c r="E119" s="28"/>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="8"/>
-      <c r="B120" s="32"/>
-      <c r="C120" s="8"/>
-      <c r="D120" s="9"/>
-      <c r="E120" s="8"/>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="8"/>
-      <c r="B121" s="32"/>
-      <c r="C121" s="8"/>
-      <c r="D121" s="9"/>
-      <c r="E121" s="8"/>
-    </row>
-    <row r="122" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="8"/>
-      <c r="B122" s="33"/>
-      <c r="C122" s="8"/>
-      <c r="D122" s="9"/>
-      <c r="E122" s="8"/>
-    </row>
-    <row r="123" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="12"/>
-      <c r="B123" s="34"/>
-      <c r="C123" s="35"/>
-      <c r="D123" s="35"/>
-      <c r="E123" s="36"/>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="13"/>
-      <c r="B124" s="31"/>
-      <c r="C124" s="13"/>
-      <c r="D124" s="14"/>
-      <c r="E124" s="28"/>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="13"/>
-      <c r="B125" s="32"/>
-      <c r="C125" s="8"/>
-      <c r="D125" s="14"/>
-      <c r="E125" s="28"/>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" s="8"/>
-      <c r="B126" s="32"/>
-      <c r="C126" s="8"/>
-      <c r="D126" s="9"/>
-      <c r="E126" s="8"/>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" s="8"/>
-      <c r="B127" s="32"/>
-      <c r="C127" s="8"/>
-      <c r="D127" s="9"/>
-      <c r="E127" s="8"/>
-    </row>
-    <row r="128" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="8"/>
-      <c r="B128" s="33"/>
-      <c r="C128" s="8"/>
-      <c r="D128" s="9"/>
-      <c r="E128" s="8"/>
-    </row>
-    <row r="129" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="12"/>
-      <c r="B129" s="34"/>
-      <c r="C129" s="35"/>
-      <c r="D129" s="35"/>
-      <c r="E129" s="36"/>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" s="13"/>
-      <c r="B130" s="31"/>
-      <c r="C130" s="13"/>
-      <c r="D130" s="14"/>
-      <c r="E130" s="28"/>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A131" s="13"/>
-      <c r="B131" s="32"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="14"/>
-      <c r="E131" s="28"/>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" s="8"/>
-      <c r="B132" s="32"/>
-      <c r="C132" s="8"/>
-      <c r="D132" s="9"/>
-      <c r="E132" s="8"/>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="8"/>
-      <c r="B133" s="32"/>
-      <c r="C133" s="8"/>
-      <c r="D133" s="9"/>
-      <c r="E133" s="8"/>
-    </row>
-    <row r="134" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="8"/>
-      <c r="B134" s="33"/>
-      <c r="C134" s="8"/>
-      <c r="D134" s="9"/>
-      <c r="E134" s="8"/>
-    </row>
-    <row r="135" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="12"/>
-      <c r="B135" s="34"/>
-      <c r="C135" s="35"/>
-      <c r="D135" s="35"/>
-      <c r="E135" s="36"/>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" s="13"/>
-      <c r="B136" s="31"/>
-      <c r="C136" s="13"/>
-      <c r="D136" s="14"/>
-      <c r="E136" s="28"/>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" s="13"/>
-      <c r="B137" s="32"/>
-      <c r="C137" s="8"/>
-      <c r="D137" s="14"/>
-      <c r="E137" s="28"/>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="8"/>
-      <c r="B138" s="32"/>
-      <c r="C138" s="8"/>
-      <c r="D138" s="9"/>
-      <c r="E138" s="8"/>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" s="8"/>
-      <c r="B139" s="32"/>
-      <c r="C139" s="8"/>
-      <c r="D139" s="9"/>
-      <c r="E139" s="8"/>
-    </row>
-    <row r="140" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="8"/>
-      <c r="B140" s="33"/>
-      <c r="C140" s="8"/>
-      <c r="D140" s="9"/>
-      <c r="E140" s="8"/>
-    </row>
-    <row r="141" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A141" s="12"/>
-      <c r="B141" s="34"/>
-      <c r="C141" s="35"/>
-      <c r="D141" s="35"/>
-      <c r="E141" s="36"/>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A142" s="13"/>
-      <c r="B142" s="31"/>
-      <c r="C142" s="13"/>
-      <c r="D142" s="14"/>
-      <c r="E142" s="28"/>
-    </row>
+      <c r="E59" s="8"/>
+    </row>
+    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="10"/>
+      <c r="B60" s="38"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="10"/>
+    </row>
+    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B61" s="27"/>
+      <c r="C61" s="15">
+        <f>MROUND(SUM(C6:C60) /60,0.2)</f>
+        <v>23.400000000000002</v>
+      </c>
+      <c r="D61" s="16"/>
+      <c r="E61" s="17"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="13"/>
-      <c r="B143" s="32"/>
-      <c r="C143" s="8"/>
+      <c r="B143" s="30"/>
+      <c r="C143" s="13"/>
       <c r="D143" s="14"/>
       <c r="E143" s="28"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A144" s="8"/>
-      <c r="B144" s="32"/>
+      <c r="A144" s="13"/>
+      <c r="B144" s="31"/>
       <c r="C144" s="8"/>
-      <c r="D144" s="9"/>
-      <c r="E144" s="8"/>
+      <c r="D144" s="14"/>
+      <c r="E144" s="28"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="8"/>
-      <c r="B145" s="32"/>
+      <c r="B145" s="31"/>
       <c r="C145" s="8"/>
       <c r="D145" s="9"/>
       <c r="E145" s="8"/>
     </row>
-    <row r="146" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="8"/>
-      <c r="B146" s="33"/>
+      <c r="B146" s="31"/>
       <c r="C146" s="8"/>
       <c r="D146" s="9"/>
       <c r="E146" s="8"/>
     </row>
     <row r="147" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="12"/>
-      <c r="B147" s="34"/>
-      <c r="C147" s="35"/>
-      <c r="D147" s="35"/>
-      <c r="E147" s="36"/>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A148" s="13"/>
-      <c r="B148" s="31"/>
-      <c r="C148" s="13"/>
-      <c r="D148" s="14"/>
-      <c r="E148" s="28"/>
+      <c r="A147" s="8"/>
+      <c r="B147" s="32"/>
+      <c r="C147" s="8"/>
+      <c r="D147" s="9"/>
+      <c r="E147" s="8"/>
+    </row>
+    <row r="148" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="12"/>
+      <c r="B148" s="33"/>
+      <c r="C148" s="34"/>
+      <c r="D148" s="34"/>
+      <c r="E148" s="35"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="13"/>
-      <c r="B149" s="32"/>
-      <c r="C149" s="8"/>
+      <c r="B149" s="30"/>
+      <c r="C149" s="13"/>
       <c r="D149" s="14"/>
       <c r="E149" s="28"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" s="8"/>
-      <c r="B150" s="32"/>
+      <c r="A150" s="13"/>
+      <c r="B150" s="31"/>
       <c r="C150" s="8"/>
-      <c r="D150" s="9"/>
-      <c r="E150" s="8"/>
+      <c r="D150" s="14"/>
+      <c r="E150" s="28"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="8"/>
-      <c r="B151" s="32"/>
+      <c r="B151" s="31"/>
       <c r="C151" s="8"/>
       <c r="D151" s="9"/>
       <c r="E151" s="8"/>
     </row>
-    <row r="152" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="8"/>
-      <c r="B152" s="33"/>
+      <c r="B152" s="31"/>
       <c r="C152" s="8"/>
       <c r="D152" s="9"/>
       <c r="E152" s="8"/>
     </row>
-    <row r="153" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="B153" s="27"/>
-      <c r="C153" s="15">
-        <f>MROUND(SUM(C6:C152) /60,0.2)</f>
-        <v>19.200000000000003</v>
-      </c>
-      <c r="D153" s="16"/>
-      <c r="E153" s="17"/>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A155" s="18" t="s">
-        <v>17</v>
-      </c>
+    <row r="153" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="8"/>
+      <c r="B153" s="32"/>
+      <c r="C153" s="8"/>
+      <c r="D153" s="9"/>
+      <c r="E153" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="53">
+  <mergeCells count="21">
+    <mergeCell ref="B56:B60"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B58:B62"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B9:E9"/>
@@ -2324,49 +1876,17 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B46:B54"/>
     <mergeCell ref="B34:B38"/>
     <mergeCell ref="B40:B44"/>
     <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:B50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:B56"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B94:B98"/>
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B100:B104"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="B106:B110"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B112:B116"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B118:B122"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B124:B128"/>
-    <mergeCell ref="B142:B146"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:B152"/>
-    <mergeCell ref="B129:E129"/>
-    <mergeCell ref="B130:B134"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B136:B140"/>
-    <mergeCell ref="B141:E141"/>
+    <mergeCell ref="B55:E55"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C52:C56 C46:C50 C40:C44 C16:C20 B6 C22:C26 C28:C32 C58:C62 C148:C152 C6:C8 C76:C80 C82:C86 C70:C74 C64:C67 C88:C92 C94:C98 C100:C104 C106:C110 C112:C116 C118:C122 C124:C128 C130:C134 C136:C140 C142:C146 C10:C14 C34:C38" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B58:B62 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B46:B50 B52:B56 B64:B68 B70:B74 B76:B80 B82:B86 B88:B92 B94:B98 B100:B104 B106:B110 B112:B116 B118:B122 B124:B128 B130:B134 B136:B140 B142:B146 B148:B152 B28:B32" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2377,7 +1897,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="28" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="40" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>

</xml_diff>

<commit_message>
chore(jdt) : maj du 28.10.26
avec quelques jours intermédiaires que je n'avait pas commit
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACCA033-32E7-4434-A191-59E17881673B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B9A04C-F3EF-4A11-A885-A8C2BA4DCB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$79</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="97">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -311,6 +311,36 @@
   </si>
   <si>
     <t>Je remplis le rapport, chapitre IA, tests, bilan produit et conception.</t>
+  </si>
+  <si>
+    <t>Corrections diverses</t>
+  </si>
+  <si>
+    <t>Corrigé le get set de Hp pour le joueur, la methode ClosestValue, quelques valeurs imprécises et commentaires.</t>
+  </si>
+  <si>
+    <t>Corrections</t>
+  </si>
+  <si>
+    <t>fait afficher Hp à 0 (avant, lorsque le joueur mourrait, il n'avait pas le temps d'afficher).</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Ajout d'un score pour le joueur.</t>
+  </si>
+  <si>
+    <t>Correction des dimensions des bales ennemies (mauvaises valeurs) et décalage des axes ennemis.</t>
+  </si>
+  <si>
+    <t>Ecran de mort</t>
+  </si>
+  <si>
+    <t>Début de l'écran de mort, faire que le jeu s'arrête en arrière plan. [WIP]</t>
+  </si>
+  <si>
+    <t>Le jeu se met en pause lorsque le joueur meurt, construction d'un écran de mort en cours.</t>
   </si>
 </sst>
 </file>
@@ -687,6 +717,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -694,30 +748,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -729,8 +759,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF66FF33"/>
       <color rgb="FFFFFFCC"/>
-      <color rgb="FF66FF33"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1036,26 +1066,26 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E153"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="107" style="1" customWidth="1"/>
-    <col min="5" max="5" width="71.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="71.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="1"/>
+    <col min="8" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="44"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -1067,10 +1097,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="44"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1082,10 +1112,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="44"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1097,12 +1127,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="47"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1121,7 +1151,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
@@ -1138,11 +1168,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="39"/>
+      <c r="B7" s="46"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1155,7 +1185,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="39"/>
+      <c r="B8" s="46"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1168,10 +1198,10 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="41"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="45"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
@@ -1192,7 +1222,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="39"/>
+      <c r="B11" s="46"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1205,7 +1235,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="39"/>
+      <c r="B12" s="46"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1218,7 +1248,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="46"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1227,11 +1257,11 @@
       </c>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="40"/>
+      <c r="B14" s="47"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1246,10 +1276,10 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="41"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="43"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="45"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -1272,7 +1302,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="39"/>
+      <c r="B17" s="46"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1285,7 +1315,7 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="39"/>
+      <c r="B18" s="46"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
@@ -1300,7 +1330,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="39"/>
+      <c r="B19" s="46"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1313,7 +1343,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="40"/>
+      <c r="B20" s="47"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1326,10 +1356,10 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="41"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="43"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="45"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
@@ -1350,7 +1380,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="39"/>
+      <c r="B23" s="46"/>
       <c r="C23" s="8">
         <v>15</v>
       </c>
@@ -1363,7 +1393,7 @@
       <c r="A24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="39"/>
+      <c r="B24" s="46"/>
       <c r="C24" s="8">
         <v>160</v>
       </c>
@@ -1374,14 +1404,14 @@
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="39"/>
+      <c r="B25" s="46"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="40"/>
+      <c r="B26" s="47"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1390,12 +1420,12 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="43"/>
-    </row>
-    <row r="28" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="43"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="45"/>
+    </row>
+    <row r="28" spans="1:5" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
@@ -1414,7 +1444,7 @@
       <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="39"/>
+      <c r="B29" s="46"/>
       <c r="C29" s="8">
         <v>70</v>
       </c>
@@ -1427,7 +1457,7 @@
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="39"/>
+      <c r="B30" s="46"/>
       <c r="C30" s="8">
         <v>10</v>
       </c>
@@ -1438,14 +1468,14 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="39"/>
+      <c r="B31" s="46"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="40"/>
+      <c r="B32" s="47"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1454,10 +1484,10 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="41"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="43"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="45"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
@@ -1478,7 +1508,7 @@
       <c r="A35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="39"/>
+      <c r="B35" s="46"/>
       <c r="C35" s="5">
         <v>160</v>
       </c>
@@ -1491,7 +1521,7 @@
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="39"/>
+      <c r="B36" s="46"/>
       <c r="C36" s="8">
         <v>5</v>
       </c>
@@ -1504,7 +1534,7 @@
       <c r="A37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="39"/>
+      <c r="B37" s="46"/>
       <c r="C37" s="8">
         <v>15</v>
       </c>
@@ -1517,7 +1547,7 @@
       <c r="A38" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="40"/>
+      <c r="B38" s="47"/>
       <c r="C38" s="10">
         <v>20</v>
       </c>
@@ -1530,10 +1560,10 @@
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="41"/>
-      <c r="C39" s="42"/>
-      <c r="D39" s="42"/>
-      <c r="E39" s="43"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="45"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
@@ -1554,7 +1584,7 @@
       <c r="A41" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="39"/>
+      <c r="B41" s="46"/>
       <c r="C41" s="8">
         <v>45</v>
       </c>
@@ -1567,7 +1597,7 @@
       <c r="A42" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="39"/>
+      <c r="B42" s="46"/>
       <c r="C42" s="8">
         <v>20</v>
       </c>
@@ -1578,14 +1608,14 @@
     </row>
     <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="39"/>
+      <c r="B43" s="46"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="40"/>
+      <c r="B44" s="47"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
@@ -1594,10 +1624,10 @@
       <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="41"/>
-      <c r="C45" s="42"/>
-      <c r="D45" s="42"/>
-      <c r="E45" s="43"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="44"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="45"/>
     </row>
     <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
@@ -1716,16 +1746,24 @@
       <c r="A55" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B55" s="41"/>
-      <c r="C55" s="42"/>
-      <c r="D55" s="42"/>
-      <c r="E55" s="43"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
-      <c r="B56" s="36"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="6"/>
+      <c r="A56" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B56" s="36">
+        <v>46321</v>
+      </c>
+      <c r="C56" s="5">
+        <v>100</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>88</v>
+      </c>
       <c r="E56" s="28"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1757,30 +1795,188 @@
       <c r="E60" s="10"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="26" t="s">
+      <c r="A61" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B61" s="43"/>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="45"/>
+    </row>
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62" s="36">
+        <v>46322</v>
+      </c>
+      <c r="C62" s="5">
+        <v>10</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E62" s="28"/>
+    </row>
+    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63" s="37"/>
+      <c r="C63" s="8">
+        <v>15</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="E63" s="28"/>
+    </row>
+    <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B64" s="37"/>
+      <c r="C64" s="8">
+        <v>30</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E64" s="8"/>
+    </row>
+    <row r="65" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B65" s="37"/>
+      <c r="C65" s="8">
+        <v>10</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E65" s="8"/>
+    </row>
+    <row r="66" spans="1:5" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="10"/>
+      <c r="B66" s="38"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="11"/>
+      <c r="E66" s="10"/>
+    </row>
+    <row r="67" spans="1:5" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B67" s="43"/>
+      <c r="C67" s="44"/>
+      <c r="D67" s="44"/>
+      <c r="E67" s="45"/>
+    </row>
+    <row r="68" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B68" s="36">
+        <v>46323</v>
+      </c>
+      <c r="C68" s="5">
+        <v>45</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E68" s="28"/>
+    </row>
+    <row r="69" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="37"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="28"/>
+    </row>
+    <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="7"/>
+      <c r="B70" s="37"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="8"/>
+    </row>
+    <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="7"/>
+      <c r="B71" s="37"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="8"/>
+    </row>
+    <row r="72" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="10"/>
+      <c r="B72" s="38"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="11"/>
+      <c r="E72" s="10"/>
+    </row>
+    <row r="73" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B73" s="43"/>
+      <c r="C73" s="44"/>
+      <c r="D73" s="44"/>
+      <c r="E73" s="45"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="4"/>
+      <c r="B74" s="36"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="6"/>
+      <c r="E74" s="28"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="7"/>
+      <c r="B75" s="37"/>
+      <c r="C75" s="8"/>
+      <c r="D75" s="9"/>
+      <c r="E75" s="28"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="7"/>
+      <c r="B76" s="37"/>
+      <c r="C76" s="8"/>
+      <c r="D76" s="9"/>
+      <c r="E76" s="8"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="7"/>
+      <c r="B77" s="37"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="8"/>
+    </row>
+    <row r="78" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="10"/>
+      <c r="B78" s="38"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="11"/>
+      <c r="E78" s="10"/>
+    </row>
+    <row r="79" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B61" s="27"/>
-      <c r="C61" s="15">
+      <c r="B79" s="27"/>
+      <c r="C79" s="15">
         <f>MROUND(SUM(C6:C60) /60,0.2)</f>
-        <v>23.400000000000002</v>
-      </c>
-      <c r="D61" s="16"/>
-      <c r="E61" s="17"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" s="16"/>
+      <c r="E79" s="17"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="142" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="13"/>
       <c r="B143" s="30"/>
@@ -1809,14 +2005,14 @@
       <c r="D146" s="9"/>
       <c r="E146" s="8"/>
     </row>
-    <row r="147" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="8"/>
       <c r="B147" s="32"/>
       <c r="C147" s="8"/>
       <c r="D147" s="9"/>
       <c r="E147" s="8"/>
     </row>
-    <row r="148" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="12"/>
       <c r="B148" s="33"/>
       <c r="C148" s="34"/>
@@ -1851,7 +2047,7 @@
       <c r="D152" s="9"/>
       <c r="E152" s="8"/>
     </row>
-    <row r="153" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="8"/>
       <c r="B153" s="32"/>
       <c r="C153" s="8"/>
@@ -1859,7 +2055,18 @@
       <c r="E153" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="27">
+    <mergeCell ref="B74:B78"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B55:E55"/>
     <mergeCell ref="B56:B60"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1876,17 +2083,12 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B55:E55"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56 B62 B68 B74" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -1915,6 +2117,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -2096,15 +2307,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -2122,6 +2324,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2137,12 +2347,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : décalage cases
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B9A04C-F3EF-4A11-A885-A8C2BA4DCB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FF0481-8C42-4523-A9D7-33E9ACF75872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$79</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$85</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -341,6 +341,9 @@
   </si>
   <si>
     <t>Le jeu se met en pause lorsque le joueur meurt, construction d'un écran de mort en cours.</t>
+  </si>
+  <si>
+    <t>L'écran de mort est fait, le jeu se met en pause et il peut se remettre en marche avec "Rejouer".</t>
   </si>
 </sst>
 </file>
@@ -1889,9 +1892,16 @@
       <c r="E68" s="28"/>
     </row>
     <row r="69" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>94</v>
+      </c>
       <c r="B69" s="37"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="9"/>
+      <c r="C69" s="8">
+        <v>90</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>97</v>
+      </c>
       <c r="E69" s="28"/>
     </row>
     <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1909,7 +1919,7 @@
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="10"/>
+      <c r="A72" s="7"/>
       <c r="B72" s="38"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
@@ -1926,7 +1936,9 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="4"/>
-      <c r="B74" s="36"/>
+      <c r="B74" s="36">
+        <v>46324</v>
+      </c>
       <c r="C74" s="5"/>
       <c r="D74" s="6"/>
       <c r="E74" s="28"/>
@@ -1959,20 +1971,64 @@
       <c r="D78" s="11"/>
       <c r="E78" s="10"/>
     </row>
-    <row r="79" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="26" t="s">
+    <row r="79" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B79" s="43"/>
+      <c r="C79" s="44"/>
+      <c r="D79" s="44"/>
+      <c r="E79" s="45"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="4"/>
+      <c r="B80" s="36"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="6"/>
+      <c r="E80" s="28"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="7"/>
+      <c r="B81" s="37"/>
+      <c r="C81" s="8"/>
+      <c r="D81" s="9"/>
+      <c r="E81" s="28"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="7"/>
+      <c r="B82" s="37"/>
+      <c r="C82" s="8"/>
+      <c r="D82" s="9"/>
+      <c r="E82" s="8"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="7"/>
+      <c r="B83" s="37"/>
+      <c r="C83" s="8"/>
+      <c r="D83" s="9"/>
+      <c r="E83" s="8"/>
+    </row>
+    <row r="84" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="10"/>
+      <c r="B84" s="38"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="11"/>
+      <c r="E84" s="10"/>
+    </row>
+    <row r="85" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B79" s="27"/>
-      <c r="C79" s="15">
+      <c r="B85" s="27"/>
+      <c r="C85" s="15">
         <f>MROUND(SUM(C6:C60) /60,0.2)</f>
         <v>25</v>
       </c>
-      <c r="D79" s="16"/>
-      <c r="E79" s="17"/>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" s="18" t="s">
+      <c r="D85" s="16"/>
+      <c r="E85" s="17"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="18" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2055,7 +2111,9 @@
       <c r="E153" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B80:B84"/>
     <mergeCell ref="B74:B78"/>
     <mergeCell ref="B61:E61"/>
     <mergeCell ref="B62:B66"/>
@@ -2085,10 +2143,10 @@
     <mergeCell ref="B33:E33"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78 C80:C84" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56 B62 B68 B74" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56 B62 B68 B74 B80" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2109,14 +2167,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2125,7 +2175,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -2307,23 +2357,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2331,7 +2373,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2347,4 +2389,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : maj du 30.10.26 (laptop)
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FF0481-8C42-4523-A9D7-33E9ACF75872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D681544-6281-40C3-9EEF-129C7C852189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$85</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$88</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="103">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -345,12 +345,27 @@
   <si>
     <t>L'écran de mort est fait, le jeu se met en pause et il peut se remettre en marche avec "Rejouer".</t>
   </si>
+  <si>
+    <t>Coms</t>
+  </si>
+  <si>
+    <t>J'ajoute des commentaires.</t>
+  </si>
+  <si>
+    <t>PlayerHp</t>
+  </si>
+  <si>
+    <t>Je remplace playerHp par une barre de vie au lieu du texte.</t>
+  </si>
+  <si>
+    <t>Il me semble que le bouton rejouer cause des exception</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Century Gothic"/>
@@ -406,6 +421,13 @@
       <name val="Century Gothic"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -589,7 +611,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -708,6 +730,18 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -720,6 +754,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -732,26 +774,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -1085,10 +1108,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="39"/>
+      <c r="C1" s="44"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -1100,10 +1123,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="39"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1115,10 +1138,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="39"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1130,12 +1153,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1158,7 +1181,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="39">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1175,7 +1198,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="46"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1188,7 +1211,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="46"/>
+      <c r="B8" s="42"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1201,16 +1224,16 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="43"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="45"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="38"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="39">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1225,7 +1248,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="46"/>
+      <c r="B11" s="42"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1238,7 +1261,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="46"/>
+      <c r="B12" s="42"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1251,7 +1274,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="46"/>
+      <c r="B13" s="42"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1264,7 +1287,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="47"/>
+      <c r="B14" s="43"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1279,16 +1302,16 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="43"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="45"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="38"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="36">
+      <c r="B16" s="39">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1305,7 +1328,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="46"/>
+      <c r="B17" s="42"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1318,7 +1341,7 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="46"/>
+      <c r="B18" s="42"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
@@ -1333,7 +1356,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="46"/>
+      <c r="B19" s="42"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1346,7 +1369,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="47"/>
+      <c r="B20" s="43"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1359,16 +1382,16 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="45"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="38"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>320</v>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="39">
         <v>46297</v>
       </c>
       <c r="C22" s="5">
@@ -1383,7 +1406,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="46"/>
+      <c r="B23" s="42"/>
       <c r="C23" s="8">
         <v>15</v>
       </c>
@@ -1396,7 +1419,7 @@
       <c r="A24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="46"/>
+      <c r="B24" s="42"/>
       <c r="C24" s="8">
         <v>160</v>
       </c>
@@ -1407,14 +1430,14 @@
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="46"/>
+      <c r="B25" s="42"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="47"/>
+      <c r="B26" s="43"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1423,16 +1446,16 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="45"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="38"/>
     </row>
     <row r="28" spans="1:5" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="36">
+      <c r="B28" s="39">
         <v>46299</v>
       </c>
       <c r="C28" s="13">
@@ -1447,7 +1470,7 @@
       <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="46"/>
+      <c r="B29" s="42"/>
       <c r="C29" s="8">
         <v>70</v>
       </c>
@@ -1460,7 +1483,7 @@
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="46"/>
+      <c r="B30" s="42"/>
       <c r="C30" s="8">
         <v>10</v>
       </c>
@@ -1471,14 +1494,14 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="46"/>
+      <c r="B31" s="42"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="47"/>
+      <c r="B32" s="43"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1487,16 +1510,16 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="43"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="45"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="38"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="36">
+      <c r="B34" s="39">
         <v>46304</v>
       </c>
       <c r="C34" s="5">
@@ -1511,7 +1534,7 @@
       <c r="A35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="46"/>
+      <c r="B35" s="42"/>
       <c r="C35" s="5">
         <v>160</v>
       </c>
@@ -1524,7 +1547,7 @@
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="46"/>
+      <c r="B36" s="42"/>
       <c r="C36" s="8">
         <v>5</v>
       </c>
@@ -1537,7 +1560,7 @@
       <c r="A37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="46"/>
+      <c r="B37" s="42"/>
       <c r="C37" s="8">
         <v>15</v>
       </c>
@@ -1550,7 +1573,7 @@
       <c r="A38" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="47"/>
+      <c r="B38" s="43"/>
       <c r="C38" s="10">
         <v>20</v>
       </c>
@@ -1563,16 +1586,16 @@
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="43"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="44"/>
-      <c r="E39" s="45"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="38"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="36">
+      <c r="B40" s="39">
         <v>46305</v>
       </c>
       <c r="C40" s="5">
@@ -1587,7 +1610,7 @@
       <c r="A41" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="46"/>
+      <c r="B41" s="42"/>
       <c r="C41" s="8">
         <v>45</v>
       </c>
@@ -1600,7 +1623,7 @@
       <c r="A42" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="46"/>
+      <c r="B42" s="42"/>
       <c r="C42" s="8">
         <v>20</v>
       </c>
@@ -1611,14 +1634,14 @@
     </row>
     <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="46"/>
+      <c r="B43" s="42"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="47"/>
+      <c r="B44" s="43"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
@@ -1627,16 +1650,16 @@
       <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="43"/>
-      <c r="C45" s="44"/>
-      <c r="D45" s="44"/>
-      <c r="E45" s="45"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B46" s="36">
+      <c r="B46" s="39">
         <v>46306</v>
       </c>
       <c r="C46" s="5">
@@ -1651,7 +1674,7 @@
       <c r="A47" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B47" s="37"/>
+      <c r="B47" s="40"/>
       <c r="C47" s="8">
         <v>40</v>
       </c>
@@ -1664,7 +1687,7 @@
       <c r="A48" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="37"/>
+      <c r="B48" s="40"/>
       <c r="C48" s="8">
         <v>40</v>
       </c>
@@ -1677,7 +1700,7 @@
       <c r="A49" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="37"/>
+      <c r="B49" s="40"/>
       <c r="C49" s="8">
         <v>70</v>
       </c>
@@ -1690,7 +1713,7 @@
       <c r="A50" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B50" s="37"/>
+      <c r="B50" s="40"/>
       <c r="C50" s="10">
         <v>15</v>
       </c>
@@ -1703,7 +1726,7 @@
       <c r="A51" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="37"/>
+      <c r="B51" s="40"/>
       <c r="C51" s="10">
         <v>20</v>
       </c>
@@ -1716,7 +1739,7 @@
       <c r="A52" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B52" s="37"/>
+      <c r="B52" s="40"/>
       <c r="C52" s="10">
         <v>20</v>
       </c>
@@ -1729,7 +1752,7 @@
       <c r="A53" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="37"/>
+      <c r="B53" s="40"/>
       <c r="C53" s="10">
         <v>30</v>
       </c>
@@ -1740,7 +1763,7 @@
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="10"/>
-      <c r="B54" s="38"/>
+      <c r="B54" s="41"/>
       <c r="C54" s="10"/>
       <c r="D54" s="11"/>
       <c r="E54" s="10"/>
@@ -1749,16 +1772,16 @@
       <c r="A55" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B55" s="43"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="36"/>
+      <c r="C55" s="37"/>
+      <c r="D55" s="37"/>
+      <c r="E55" s="38"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B56" s="36">
+      <c r="B56" s="39">
         <v>46321</v>
       </c>
       <c r="C56" s="5">
@@ -1771,28 +1794,28 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="37"/>
+      <c r="B57" s="40"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="28"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="37"/>
+      <c r="B58" s="40"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="37"/>
+      <c r="B59" s="40"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="10"/>
-      <c r="B60" s="38"/>
+      <c r="B60" s="41"/>
       <c r="C60" s="10"/>
       <c r="D60" s="11"/>
       <c r="E60" s="10"/>
@@ -1801,16 +1824,16 @@
       <c r="A61" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B61" s="43"/>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="45"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="37"/>
+      <c r="D61" s="37"/>
+      <c r="E61" s="38"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B62" s="36">
+      <c r="B62" s="39">
         <v>46322</v>
       </c>
       <c r="C62" s="5">
@@ -1825,7 +1848,7 @@
       <c r="A63" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B63" s="37"/>
+      <c r="B63" s="40"/>
       <c r="C63" s="8">
         <v>15</v>
       </c>
@@ -1838,7 +1861,7 @@
       <c r="A64" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B64" s="37"/>
+      <c r="B64" s="40"/>
       <c r="C64" s="8">
         <v>30</v>
       </c>
@@ -1851,7 +1874,7 @@
       <c r="A65" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B65" s="37"/>
+      <c r="B65" s="40"/>
       <c r="C65" s="8">
         <v>10</v>
       </c>
@@ -1862,7 +1885,7 @@
     </row>
     <row r="66" spans="1:5" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="38"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -1871,16 +1894,16 @@
       <c r="A67" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B67" s="43"/>
-      <c r="C67" s="44"/>
-      <c r="D67" s="44"/>
-      <c r="E67" s="45"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="37"/>
+      <c r="D67" s="37"/>
+      <c r="E67" s="38"/>
     </row>
     <row r="68" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B68" s="36">
+      <c r="B68" s="39">
         <v>46323</v>
       </c>
       <c r="C68" s="5">
@@ -1895,7 +1918,7 @@
       <c r="A69" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B69" s="37"/>
+      <c r="B69" s="40"/>
       <c r="C69" s="8">
         <v>90</v>
       </c>
@@ -1906,21 +1929,21 @@
     </row>
     <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="37"/>
+      <c r="B70" s="40"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="37"/>
+      <c r="B71" s="40"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="7"/>
-      <c r="B72" s="38"/>
+      <c r="B72" s="41"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -1929,14 +1952,14 @@
       <c r="A73" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B73" s="43"/>
-      <c r="C73" s="44"/>
-      <c r="D73" s="44"/>
-      <c r="E73" s="45"/>
+      <c r="B73" s="36"/>
+      <c r="C73" s="37"/>
+      <c r="D73" s="37"/>
+      <c r="E73" s="38"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="4"/>
-      <c r="B74" s="36">
+      <c r="B74" s="39">
         <v>46324</v>
       </c>
       <c r="C74" s="5"/>
@@ -1945,28 +1968,28 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="7"/>
-      <c r="B75" s="37"/>
+      <c r="B75" s="40"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="28"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
-      <c r="B76" s="37"/>
+      <c r="B76" s="40"/>
       <c r="C76" s="8"/>
       <c r="D76" s="9"/>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="37"/>
+      <c r="B77" s="40"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="10"/>
-      <c r="B78" s="38"/>
+      <c r="B78" s="41"/>
       <c r="C78" s="10"/>
       <c r="D78" s="11"/>
       <c r="E78" s="10"/>
@@ -1975,60 +1998,96 @@
       <c r="A79" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B79" s="43"/>
-      <c r="C79" s="44"/>
-      <c r="D79" s="44"/>
-      <c r="E79" s="45"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="37"/>
+      <c r="D79" s="37"/>
+      <c r="E79" s="38"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="4"/>
-      <c r="B80" s="36"/>
-      <c r="C80" s="5"/>
-      <c r="D80" s="6"/>
+      <c r="A80" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B80" s="39">
+        <v>46325</v>
+      </c>
+      <c r="C80" s="5">
+        <v>5</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="E80" s="28"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="7"/>
-      <c r="B81" s="37"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="9"/>
-      <c r="E81" s="28"/>
+      <c r="A81" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B81" s="40"/>
+      <c r="C81" s="8">
+        <v>15</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="7"/>
-      <c r="B82" s="37"/>
+      <c r="B82" s="40"/>
       <c r="C82" s="8"/>
-      <c r="D82" s="9"/>
+      <c r="D82" s="48" t="s">
+        <v>102</v>
+      </c>
       <c r="E82" s="8"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="7"/>
-      <c r="B83" s="37"/>
+      <c r="B83" s="40"/>
       <c r="C83" s="8"/>
       <c r="D83" s="9"/>
       <c r="E83" s="8"/>
     </row>
-    <row r="84" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
-      <c r="B84" s="38"/>
+      <c r="B84" s="40"/>
       <c r="C84" s="10"/>
       <c r="D84" s="11"/>
       <c r="E84" s="10"/>
     </row>
-    <row r="85" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="26" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="7"/>
+      <c r="B85" s="40"/>
+      <c r="C85" s="8"/>
+      <c r="D85" s="9"/>
+      <c r="E85" s="8"/>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="7"/>
+      <c r="B86" s="40"/>
+      <c r="C86" s="8"/>
+      <c r="D86" s="9"/>
+      <c r="E86" s="8"/>
+    </row>
+    <row r="87" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="10"/>
+      <c r="B87" s="41"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="11"/>
+      <c r="E87" s="10"/>
+    </row>
+    <row r="88" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B85" s="27"/>
-      <c r="C85" s="15">
+      <c r="B88" s="27"/>
+      <c r="C88" s="15">
         <f>MROUND(SUM(C6:C60) /60,0.2)</f>
         <v>25</v>
       </c>
-      <c r="D85" s="16"/>
-      <c r="E85" s="17"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="18" t="s">
+      <c r="D88" s="16"/>
+      <c r="E88" s="17"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="18" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2112,19 +2171,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B80:B84"/>
-    <mergeCell ref="B74:B78"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B55:E55"/>
     <mergeCell ref="B56:B60"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -2141,9 +2187,22 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B74:B78"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B80:B87"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78 C80:C84" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78 C80:C87" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56 B62 B68 B74 B80" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
@@ -2167,15 +2226,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100735015723C2CFE488EA62BE6EBA752B5" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="879a0952b67ddc4861aa98f664a08e07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0dcbab57-ce0d-48ec-9006-afbf43b82b42" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="872bcaed78208874ee82016f6206aa40" ns3:_="">
     <xsd:import namespace="0dcbab57-ce0d-48ec-9006-afbf43b82b42"/>
@@ -2357,6 +2407,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2366,14 +2425,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B770EEE6-8508-4E91-92ED-FD5AB7F9B972}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2387,6 +2438,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
chore(doc) : maj 30.10 intermediaire
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D681544-6281-40C3-9EEF-129C7C852189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C96DE0-DC4D-4DF9-B27C-4286728A1589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="107">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -358,14 +358,27 @@
     <t>Je remplace playerHp par une barre de vie au lieu du texte.</t>
   </si>
   <si>
-    <t>Il me semble que le bouton rejouer cause des exception</t>
+    <t>Config</t>
+  </si>
+  <si>
+    <t>J'ai enlevé de Config les constantes qui étaient propres à une classe,
+passant donc de Config.GOUVERNAIL_SPEED à Gouvernail.SPEED par ex</t>
+  </si>
+  <si>
+    <t>rejouer</t>
+  </si>
+  <si>
+    <t>Je change quelques lignes qui causaient une stack overflow exception lors de "rejouer"</t>
+  </si>
+  <si>
+    <t>meilleurScore</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Century Gothic"/>
@@ -421,13 +434,6 @@
       <name val="Century Gothic"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Century Gothic"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -730,6 +736,30 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -742,18 +772,6 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -762,19 +780,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -1092,26 +1100,26 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E153"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="107" style="1" customWidth="1"/>
-    <col min="5" max="5" width="71.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="71.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.44140625" style="1"/>
+    <col min="8" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="44"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -1123,10 +1131,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="44"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1138,10 +1146,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="44"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1153,12 +1161,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="47"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1177,11 +1185,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="36">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1194,11 +1202,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="42"/>
+      <c r="B7" s="46"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1211,7 +1219,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="42"/>
+      <c r="B8" s="46"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1224,16 +1232,16 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="38"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="45"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="39">
+      <c r="B10" s="36">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1248,7 +1256,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="42"/>
+      <c r="B11" s="46"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1261,7 +1269,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="42"/>
+      <c r="B12" s="46"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1274,7 +1282,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="42"/>
+      <c r="B13" s="46"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1283,11 +1291,11 @@
       </c>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="43"/>
+      <c r="B14" s="47"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1302,16 +1310,16 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="38"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="45"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="39">
+      <c r="B16" s="36">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1328,7 +1336,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="42"/>
+      <c r="B17" s="46"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1341,7 +1349,7 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="42"/>
+      <c r="B18" s="46"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
@@ -1356,7 +1364,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="42"/>
+      <c r="B19" s="46"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1369,7 +1377,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="43"/>
+      <c r="B20" s="47"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1382,16 +1390,16 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="45"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>320</v>
       </c>
-      <c r="B22" s="39">
+      <c r="B22" s="36">
         <v>46297</v>
       </c>
       <c r="C22" s="5">
@@ -1406,7 +1414,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="42"/>
+      <c r="B23" s="46"/>
       <c r="C23" s="8">
         <v>15</v>
       </c>
@@ -1419,7 +1427,7 @@
       <c r="A24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="42"/>
+      <c r="B24" s="46"/>
       <c r="C24" s="8">
         <v>160</v>
       </c>
@@ -1430,14 +1438,14 @@
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="42"/>
+      <c r="B25" s="46"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="43"/>
+      <c r="B26" s="47"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1446,16 +1454,16 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38"/>
-    </row>
-    <row r="28" spans="1:5" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="43"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="45"/>
+    </row>
+    <row r="28" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="39">
+      <c r="B28" s="36">
         <v>46299</v>
       </c>
       <c r="C28" s="13">
@@ -1470,7 +1478,7 @@
       <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="42"/>
+      <c r="B29" s="46"/>
       <c r="C29" s="8">
         <v>70</v>
       </c>
@@ -1483,7 +1491,7 @@
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="42"/>
+      <c r="B30" s="46"/>
       <c r="C30" s="8">
         <v>10</v>
       </c>
@@ -1494,14 +1502,14 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="42"/>
+      <c r="B31" s="46"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="43"/>
+      <c r="B32" s="47"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1510,16 +1518,16 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="36"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="38"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="45"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="39">
+      <c r="B34" s="36">
         <v>46304</v>
       </c>
       <c r="C34" s="5">
@@ -1534,7 +1542,7 @@
       <c r="A35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="42"/>
+      <c r="B35" s="46"/>
       <c r="C35" s="5">
         <v>160</v>
       </c>
@@ -1547,7 +1555,7 @@
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="42"/>
+      <c r="B36" s="46"/>
       <c r="C36" s="8">
         <v>5</v>
       </c>
@@ -1560,7 +1568,7 @@
       <c r="A37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="42"/>
+      <c r="B37" s="46"/>
       <c r="C37" s="8">
         <v>15</v>
       </c>
@@ -1573,7 +1581,7 @@
       <c r="A38" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="43"/>
+      <c r="B38" s="47"/>
       <c r="C38" s="10">
         <v>20</v>
       </c>
@@ -1586,16 +1594,16 @@
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="36"/>
-      <c r="C39" s="37"/>
-      <c r="D39" s="37"/>
-      <c r="E39" s="38"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="45"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="39">
+      <c r="B40" s="36">
         <v>46305</v>
       </c>
       <c r="C40" s="5">
@@ -1610,7 +1618,7 @@
       <c r="A41" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="42"/>
+      <c r="B41" s="46"/>
       <c r="C41" s="8">
         <v>45</v>
       </c>
@@ -1623,7 +1631,7 @@
       <c r="A42" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="42"/>
+      <c r="B42" s="46"/>
       <c r="C42" s="8">
         <v>20</v>
       </c>
@@ -1634,14 +1642,14 @@
     </row>
     <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="42"/>
+      <c r="B43" s="46"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="43"/>
+      <c r="B44" s="47"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
@@ -1650,16 +1658,16 @@
       <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="36"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="44"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="45"/>
     </row>
     <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B46" s="39">
+      <c r="B46" s="36">
         <v>46306</v>
       </c>
       <c r="C46" s="5">
@@ -1674,7 +1682,7 @@
       <c r="A47" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B47" s="40"/>
+      <c r="B47" s="37"/>
       <c r="C47" s="8">
         <v>40</v>
       </c>
@@ -1687,7 +1695,7 @@
       <c r="A48" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="40"/>
+      <c r="B48" s="37"/>
       <c r="C48" s="8">
         <v>40</v>
       </c>
@@ -1700,7 +1708,7 @@
       <c r="A49" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="40"/>
+      <c r="B49" s="37"/>
       <c r="C49" s="8">
         <v>70</v>
       </c>
@@ -1713,7 +1721,7 @@
       <c r="A50" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B50" s="40"/>
+      <c r="B50" s="37"/>
       <c r="C50" s="10">
         <v>15</v>
       </c>
@@ -1726,7 +1734,7 @@
       <c r="A51" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="40"/>
+      <c r="B51" s="37"/>
       <c r="C51" s="10">
         <v>20</v>
       </c>
@@ -1739,7 +1747,7 @@
       <c r="A52" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B52" s="40"/>
+      <c r="B52" s="37"/>
       <c r="C52" s="10">
         <v>20</v>
       </c>
@@ -1752,7 +1760,7 @@
       <c r="A53" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="40"/>
+      <c r="B53" s="37"/>
       <c r="C53" s="10">
         <v>30</v>
       </c>
@@ -1763,7 +1771,7 @@
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="10"/>
-      <c r="B54" s="41"/>
+      <c r="B54" s="38"/>
       <c r="C54" s="10"/>
       <c r="D54" s="11"/>
       <c r="E54" s="10"/>
@@ -1772,16 +1780,16 @@
       <c r="A55" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B55" s="36"/>
-      <c r="C55" s="37"/>
-      <c r="D55" s="37"/>
-      <c r="E55" s="38"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="45"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B56" s="39">
+      <c r="B56" s="36">
         <v>46321</v>
       </c>
       <c r="C56" s="5">
@@ -1794,28 +1802,28 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="40"/>
+      <c r="B57" s="37"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="28"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="40"/>
+      <c r="B58" s="37"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="40"/>
+      <c r="B59" s="37"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="10"/>
-      <c r="B60" s="41"/>
+      <c r="B60" s="38"/>
       <c r="C60" s="10"/>
       <c r="D60" s="11"/>
       <c r="E60" s="10"/>
@@ -1824,16 +1832,16 @@
       <c r="A61" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B61" s="36"/>
-      <c r="C61" s="37"/>
-      <c r="D61" s="37"/>
-      <c r="E61" s="38"/>
+      <c r="B61" s="43"/>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="45"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B62" s="39">
+      <c r="B62" s="36">
         <v>46322</v>
       </c>
       <c r="C62" s="5">
@@ -1848,7 +1856,7 @@
       <c r="A63" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B63" s="40"/>
+      <c r="B63" s="37"/>
       <c r="C63" s="8">
         <v>15</v>
       </c>
@@ -1861,7 +1869,7 @@
       <c r="A64" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B64" s="40"/>
+      <c r="B64" s="37"/>
       <c r="C64" s="8">
         <v>30</v>
       </c>
@@ -1874,7 +1882,7 @@
       <c r="A65" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B65" s="40"/>
+      <c r="B65" s="37"/>
       <c r="C65" s="8">
         <v>10</v>
       </c>
@@ -1885,7 +1893,7 @@
     </row>
     <row r="66" spans="1:5" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="41"/>
+      <c r="B66" s="38"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -1894,16 +1902,16 @@
       <c r="A67" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B67" s="36"/>
-      <c r="C67" s="37"/>
-      <c r="D67" s="37"/>
-      <c r="E67" s="38"/>
-    </row>
-    <row r="68" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="43"/>
+      <c r="C67" s="44"/>
+      <c r="D67" s="44"/>
+      <c r="E67" s="45"/>
+    </row>
+    <row r="68" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B68" s="39">
+      <c r="B68" s="36">
         <v>46323</v>
       </c>
       <c r="C68" s="5">
@@ -1914,11 +1922,11 @@
       </c>
       <c r="E68" s="28"/>
     </row>
-    <row r="69" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B69" s="40"/>
+      <c r="B69" s="37"/>
       <c r="C69" s="8">
         <v>90</v>
       </c>
@@ -1929,37 +1937,37 @@
     </row>
     <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="40"/>
+      <c r="B70" s="37"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="40"/>
+      <c r="B71" s="37"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
-    <row r="72" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="7"/>
-      <c r="B72" s="41"/>
+      <c r="B72" s="38"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
     </row>
-    <row r="73" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B73" s="36"/>
-      <c r="C73" s="37"/>
-      <c r="D73" s="37"/>
-      <c r="E73" s="38"/>
+      <c r="B73" s="43"/>
+      <c r="C73" s="44"/>
+      <c r="D73" s="44"/>
+      <c r="E73" s="45"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="4"/>
-      <c r="B74" s="39">
+      <c r="B74" s="36">
         <v>46324</v>
       </c>
       <c r="C74" s="5"/>
@@ -1968,46 +1976,46 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="7"/>
-      <c r="B75" s="40"/>
+      <c r="B75" s="37"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="28"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
-      <c r="B76" s="40"/>
+      <c r="B76" s="37"/>
       <c r="C76" s="8"/>
       <c r="D76" s="9"/>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="40"/>
+      <c r="B77" s="37"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
       <c r="E77" s="8"/>
     </row>
-    <row r="78" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="10"/>
-      <c r="B78" s="41"/>
+      <c r="B78" s="38"/>
       <c r="C78" s="10"/>
       <c r="D78" s="11"/>
       <c r="E78" s="10"/>
     </row>
-    <row r="79" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B79" s="36"/>
-      <c r="C79" s="37"/>
-      <c r="D79" s="37"/>
-      <c r="E79" s="38"/>
+      <c r="B79" s="43"/>
+      <c r="C79" s="44"/>
+      <c r="D79" s="44"/>
+      <c r="E79" s="45"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B80" s="39">
+      <c r="B80" s="36">
         <v>46325</v>
       </c>
       <c r="C80" s="5">
@@ -2022,7 +2030,7 @@
       <c r="A81" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B81" s="40"/>
+      <c r="B81" s="37"/>
       <c r="C81" s="8">
         <v>15</v>
       </c>
@@ -2030,51 +2038,65 @@
         <v>101</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="7"/>
-      <c r="B82" s="40"/>
-      <c r="C82" s="8"/>
+    <row r="82" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A82" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B82" s="37"/>
+      <c r="C82" s="8">
+        <v>35</v>
+      </c>
       <c r="D82" s="48" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E82" s="8"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="7"/>
-      <c r="B83" s="40"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="9"/>
+      <c r="A83" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B83" s="37"/>
+      <c r="C83" s="8">
+        <v>20</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>105</v>
+      </c>
       <c r="E83" s="8"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="10"/>
-      <c r="B84" s="40"/>
-      <c r="C84" s="10"/>
+      <c r="A84" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B84" s="37"/>
+      <c r="C84" s="10">
+        <v>25</v>
+      </c>
       <c r="D84" s="11"/>
       <c r="E84" s="10"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="40"/>
+      <c r="B85" s="37"/>
       <c r="C85" s="8"/>
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="40"/>
+      <c r="B86" s="37"/>
       <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
-    <row r="87" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="41"/>
+      <c r="B87" s="38"/>
       <c r="C87" s="10"/>
       <c r="D87" s="11"/>
       <c r="E87" s="10"/>
     </row>
-    <row r="88" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="26" t="s">
         <v>16</v>
       </c>
@@ -2091,7 +2113,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="142" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="142" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="13"/>
       <c r="B143" s="30"/>
@@ -2120,14 +2142,14 @@
       <c r="D146" s="9"/>
       <c r="E146" s="8"/>
     </row>
-    <row r="147" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="8"/>
       <c r="B147" s="32"/>
       <c r="C147" s="8"/>
       <c r="D147" s="9"/>
       <c r="E147" s="8"/>
     </row>
-    <row r="148" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="12"/>
       <c r="B148" s="33"/>
       <c r="C148" s="34"/>
@@ -2162,7 +2184,7 @@
       <c r="D152" s="9"/>
       <c r="E152" s="8"/>
     </row>
-    <row r="153" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="8"/>
       <c r="B153" s="32"/>
       <c r="C153" s="8"/>
@@ -2171,6 +2193,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="B80:B87"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B74:B78"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B55:E55"/>
     <mergeCell ref="B56:B60"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -2187,19 +2222,6 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B74:B78"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B80:B87"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78 C80:C87" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -2216,7 +2238,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="40" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="42" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2408,20 +2430,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2443,14 +2465,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -2464,4 +2478,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore(jdt) : maj 31.10.26
</commit_message>
<xml_diff>
--- a/doc/T-P_320-pe84djb-JDT.xlsx
+++ b/doc/T-P_320-pe84djb-JDT.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pe84djb\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yohan\Documents\GitHub\Projet-320-ShootMeUp-YFS\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C96DE0-DC4D-4DF9-B27C-4286728A1589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3137BBB5-0E61-495B-80C1-522642267904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$88</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$94</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="113">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -372,6 +372,24 @@
   </si>
   <si>
     <t>meilleurScore</t>
+  </si>
+  <si>
+    <t>deathscreen</t>
+  </si>
+  <si>
+    <t>finitions, commentaires</t>
+  </si>
+  <si>
+    <t>Fin du rapport</t>
+  </si>
+  <si>
+    <t>program</t>
+  </si>
+  <si>
+    <t>Je met l'instaciation des entités comme parametre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -736,6 +754,9 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -748,6 +769,26 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -759,29 +800,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1116,10 +1134,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="39"/>
+      <c r="C1" s="45"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -1131,10 +1149,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="39"/>
+      <c r="C2" s="45"/>
       <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
@@ -1146,10 +1164,10 @@
       <c r="A3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="39"/>
+      <c r="C3" s="45"/>
       <c r="D3" s="22" t="s">
         <v>8</v>
       </c>
@@ -1161,12 +1179,12 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="48"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1189,7 +1207,7 @@
       <c r="A6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="37">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1206,7 +1224,7 @@
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="46"/>
+      <c r="B7" s="43"/>
       <c r="C7" s="8">
         <v>55</v>
       </c>
@@ -1219,7 +1237,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="46"/>
+      <c r="B8" s="43"/>
       <c r="C8" s="8">
         <v>35</v>
       </c>
@@ -1232,16 +1250,16 @@
       <c r="A9" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="43"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="45"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="42"/>
     </row>
     <row r="10" spans="1:5" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="37">
         <v>46269</v>
       </c>
       <c r="C10" s="5">
@@ -1256,7 +1274,7 @@
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="46"/>
+      <c r="B11" s="43"/>
       <c r="C11" s="8">
         <v>40</v>
       </c>
@@ -1269,7 +1287,7 @@
       <c r="A12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="46"/>
+      <c r="B12" s="43"/>
       <c r="C12" s="8">
         <v>55</v>
       </c>
@@ -1282,7 +1300,7 @@
       <c r="A13" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="46"/>
+      <c r="B13" s="43"/>
       <c r="C13" s="10">
         <v>40</v>
       </c>
@@ -1295,7 +1313,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="47"/>
+      <c r="B14" s="44"/>
       <c r="C14" s="8">
         <v>20</v>
       </c>
@@ -1310,16 +1328,16 @@
       <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="43"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="45"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="42"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="36">
+      <c r="B16" s="37">
         <v>46276</v>
       </c>
       <c r="C16" s="5">
@@ -1336,7 +1354,7 @@
       <c r="A17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="46"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="8">
         <v>10</v>
       </c>
@@ -1349,7 +1367,7 @@
       <c r="A18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="46"/>
+      <c r="B18" s="43"/>
       <c r="C18" s="8">
         <v>45</v>
       </c>
@@ -1364,7 +1382,7 @@
       <c r="A19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="46"/>
+      <c r="B19" s="43"/>
       <c r="C19" s="8">
         <v>25</v>
       </c>
@@ -1377,7 +1395,7 @@
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="47"/>
+      <c r="B20" s="44"/>
       <c r="C20" s="10">
         <v>20</v>
       </c>
@@ -1390,16 +1408,16 @@
       <c r="A21" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="45"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="42"/>
     </row>
     <row r="22" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>320</v>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="37">
         <v>46297</v>
       </c>
       <c r="C22" s="5">
@@ -1414,7 +1432,7 @@
       <c r="A23" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="46"/>
+      <c r="B23" s="43"/>
       <c r="C23" s="8">
         <v>15</v>
       </c>
@@ -1427,7 +1445,7 @@
       <c r="A24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="46"/>
+      <c r="B24" s="43"/>
       <c r="C24" s="8">
         <v>160</v>
       </c>
@@ -1438,14 +1456,14 @@
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="46"/>
+      <c r="B25" s="43"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
-      <c r="B26" s="47"/>
+      <c r="B26" s="44"/>
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="10"/>
@@ -1454,16 +1472,16 @@
       <c r="A27" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="45"/>
+      <c r="B27" s="40"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="42"/>
     </row>
     <row r="28" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="36">
+      <c r="B28" s="37">
         <v>46299</v>
       </c>
       <c r="C28" s="13">
@@ -1478,7 +1496,7 @@
       <c r="A29" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="46"/>
+      <c r="B29" s="43"/>
       <c r="C29" s="8">
         <v>70</v>
       </c>
@@ -1491,7 +1509,7 @@
       <c r="A30" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="46"/>
+      <c r="B30" s="43"/>
       <c r="C30" s="8">
         <v>10</v>
       </c>
@@ -1502,14 +1520,14 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
-      <c r="B31" s="46"/>
+      <c r="B31" s="43"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
-      <c r="B32" s="47"/>
+      <c r="B32" s="44"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
@@ -1518,16 +1536,16 @@
       <c r="A33" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="43"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="45"/>
+      <c r="B33" s="40"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="42"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="36">
+      <c r="B34" s="37">
         <v>46304</v>
       </c>
       <c r="C34" s="5">
@@ -1542,7 +1560,7 @@
       <c r="A35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="46"/>
+      <c r="B35" s="43"/>
       <c r="C35" s="5">
         <v>160</v>
       </c>
@@ -1555,7 +1573,7 @@
       <c r="A36" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="46"/>
+      <c r="B36" s="43"/>
       <c r="C36" s="8">
         <v>5</v>
       </c>
@@ -1568,7 +1586,7 @@
       <c r="A37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="46"/>
+      <c r="B37" s="43"/>
       <c r="C37" s="8">
         <v>15</v>
       </c>
@@ -1581,7 +1599,7 @@
       <c r="A38" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B38" s="47"/>
+      <c r="B38" s="44"/>
       <c r="C38" s="10">
         <v>20</v>
       </c>
@@ -1594,16 +1612,16 @@
       <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="43"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="44"/>
-      <c r="E39" s="45"/>
+      <c r="B39" s="40"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="42"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="36">
+      <c r="B40" s="37">
         <v>46305</v>
       </c>
       <c r="C40" s="5">
@@ -1618,7 +1636,7 @@
       <c r="A41" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="46"/>
+      <c r="B41" s="43"/>
       <c r="C41" s="8">
         <v>45</v>
       </c>
@@ -1631,7 +1649,7 @@
       <c r="A42" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="46"/>
+      <c r="B42" s="43"/>
       <c r="C42" s="8">
         <v>20</v>
       </c>
@@ -1642,14 +1660,14 @@
     </row>
     <row r="43" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="46"/>
+      <c r="B43" s="43"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10"/>
-      <c r="B44" s="47"/>
+      <c r="B44" s="44"/>
       <c r="C44" s="10"/>
       <c r="D44" s="11"/>
       <c r="E44" s="10"/>
@@ -1658,16 +1676,16 @@
       <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="43"/>
-      <c r="C45" s="44"/>
-      <c r="D45" s="44"/>
-      <c r="E45" s="45"/>
+      <c r="B45" s="40"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="42"/>
     </row>
     <row r="46" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B46" s="36">
+      <c r="B46" s="37">
         <v>46306</v>
       </c>
       <c r="C46" s="5">
@@ -1682,7 +1700,7 @@
       <c r="A47" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B47" s="37"/>
+      <c r="B47" s="38"/>
       <c r="C47" s="8">
         <v>40</v>
       </c>
@@ -1695,7 +1713,7 @@
       <c r="A48" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="37"/>
+      <c r="B48" s="38"/>
       <c r="C48" s="8">
         <v>40</v>
       </c>
@@ -1708,7 +1726,7 @@
       <c r="A49" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="37"/>
+      <c r="B49" s="38"/>
       <c r="C49" s="8">
         <v>70</v>
       </c>
@@ -1721,7 +1739,7 @@
       <c r="A50" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B50" s="37"/>
+      <c r="B50" s="38"/>
       <c r="C50" s="10">
         <v>15</v>
       </c>
@@ -1734,7 +1752,7 @@
       <c r="A51" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="37"/>
+      <c r="B51" s="38"/>
       <c r="C51" s="10">
         <v>20</v>
       </c>
@@ -1747,7 +1765,7 @@
       <c r="A52" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B52" s="37"/>
+      <c r="B52" s="38"/>
       <c r="C52" s="10">
         <v>20</v>
       </c>
@@ -1760,7 +1778,7 @@
       <c r="A53" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="37"/>
+      <c r="B53" s="38"/>
       <c r="C53" s="10">
         <v>30</v>
       </c>
@@ -1771,7 +1789,7 @@
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="10"/>
-      <c r="B54" s="38"/>
+      <c r="B54" s="39"/>
       <c r="C54" s="10"/>
       <c r="D54" s="11"/>
       <c r="E54" s="10"/>
@@ -1780,16 +1798,16 @@
       <c r="A55" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B55" s="43"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="44"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="40"/>
+      <c r="C55" s="41"/>
+      <c r="D55" s="41"/>
+      <c r="E55" s="42"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B56" s="36">
+      <c r="B56" s="37">
         <v>46321</v>
       </c>
       <c r="C56" s="5">
@@ -1802,28 +1820,28 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="37"/>
+      <c r="B57" s="38"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="28"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="37"/>
+      <c r="B58" s="38"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="37"/>
+      <c r="B59" s="38"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="10"/>
-      <c r="B60" s="38"/>
+      <c r="B60" s="39"/>
       <c r="C60" s="10"/>
       <c r="D60" s="11"/>
       <c r="E60" s="10"/>
@@ -1832,16 +1850,16 @@
       <c r="A61" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B61" s="43"/>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="45"/>
+      <c r="B61" s="40"/>
+      <c r="C61" s="41"/>
+      <c r="D61" s="41"/>
+      <c r="E61" s="42"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B62" s="36">
+      <c r="B62" s="37">
         <v>46322</v>
       </c>
       <c r="C62" s="5">
@@ -1856,7 +1874,7 @@
       <c r="A63" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B63" s="37"/>
+      <c r="B63" s="38"/>
       <c r="C63" s="8">
         <v>15</v>
       </c>
@@ -1869,7 +1887,7 @@
       <c r="A64" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B64" s="37"/>
+      <c r="B64" s="38"/>
       <c r="C64" s="8">
         <v>30</v>
       </c>
@@ -1882,7 +1900,7 @@
       <c r="A65" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B65" s="37"/>
+      <c r="B65" s="38"/>
       <c r="C65" s="8">
         <v>10</v>
       </c>
@@ -1893,7 +1911,7 @@
     </row>
     <row r="66" spans="1:5" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="38"/>
+      <c r="B66" s="39"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -1902,16 +1920,16 @@
       <c r="A67" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B67" s="43"/>
-      <c r="C67" s="44"/>
-      <c r="D67" s="44"/>
-      <c r="E67" s="45"/>
+      <c r="B67" s="40"/>
+      <c r="C67" s="41"/>
+      <c r="D67" s="41"/>
+      <c r="E67" s="42"/>
     </row>
     <row r="68" spans="1:5" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B68" s="36">
+      <c r="B68" s="37">
         <v>46323</v>
       </c>
       <c r="C68" s="5">
@@ -1926,7 +1944,7 @@
       <c r="A69" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B69" s="37"/>
+      <c r="B69" s="38"/>
       <c r="C69" s="8">
         <v>90</v>
       </c>
@@ -1937,21 +1955,21 @@
     </row>
     <row r="70" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="37"/>
+      <c r="B70" s="38"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="37"/>
+      <c r="B71" s="38"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="7"/>
-      <c r="B72" s="38"/>
+      <c r="B72" s="39"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -1960,44 +1978,50 @@
       <c r="A73" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B73" s="43"/>
-      <c r="C73" s="44"/>
-      <c r="D73" s="44"/>
-      <c r="E73" s="45"/>
+      <c r="B73" s="40"/>
+      <c r="C73" s="41"/>
+      <c r="D73" s="41"/>
+      <c r="E73" s="42"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="4"/>
-      <c r="B74" s="36">
+      <c r="A74" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B74" s="37">
         <v>46324</v>
       </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="6"/>
+      <c r="C74" s="5">
+        <v>20</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>108</v>
+      </c>
       <c r="E74" s="28"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="7"/>
-      <c r="B75" s="37"/>
+      <c r="B75" s="38"/>
       <c r="C75" s="8"/>
       <c r="D75" s="9"/>
       <c r="E75" s="28"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="7"/>
-      <c r="B76" s="37"/>
+      <c r="B76" s="38"/>
       <c r="C76" s="8"/>
       <c r="D76" s="9"/>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="37"/>
+      <c r="B77" s="38"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="10"/>
-      <c r="B78" s="38"/>
+      <c r="B78" s="39"/>
       <c r="C78" s="10"/>
       <c r="D78" s="11"/>
       <c r="E78" s="10"/>
@@ -2006,16 +2030,16 @@
       <c r="A79" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B79" s="43"/>
-      <c r="C79" s="44"/>
-      <c r="D79" s="44"/>
-      <c r="E79" s="45"/>
+      <c r="B79" s="40"/>
+      <c r="C79" s="41"/>
+      <c r="D79" s="41"/>
+      <c r="E79" s="42"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B80" s="36">
+      <c r="B80" s="37">
         <v>46325</v>
       </c>
       <c r="C80" s="5">
@@ -2030,7 +2054,7 @@
       <c r="A81" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B81" s="37"/>
+      <c r="B81" s="38"/>
       <c r="C81" s="8">
         <v>15</v>
       </c>
@@ -2042,11 +2066,11 @@
       <c r="A82" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B82" s="37"/>
+      <c r="B82" s="38"/>
       <c r="C82" s="8">
         <v>35</v>
       </c>
-      <c r="D82" s="48" t="s">
+      <c r="D82" s="36" t="s">
         <v>103</v>
       </c>
       <c r="E82" s="8"/>
@@ -2055,7 +2079,7 @@
       <c r="A83" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B83" s="37"/>
+      <c r="B83" s="38"/>
       <c r="C83" s="8">
         <v>20</v>
       </c>
@@ -2068,7 +2092,7 @@
       <c r="A84" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="B84" s="37"/>
+      <c r="B84" s="38"/>
       <c r="C84" s="10">
         <v>25</v>
       </c>
@@ -2077,39 +2101,99 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="37"/>
+      <c r="B85" s="38"/>
       <c r="C85" s="8"/>
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="37"/>
+      <c r="B86" s="38"/>
       <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="38"/>
+      <c r="B87" s="39"/>
       <c r="C87" s="10"/>
       <c r="D87" s="11"/>
       <c r="E87" s="10"/>
     </row>
-    <row r="88" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="26" t="s">
+    <row r="88" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B88" s="40"/>
+      <c r="C88" s="41"/>
+      <c r="D88" s="41"/>
+      <c r="E88" s="42"/>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B89" s="37">
+        <v>46326</v>
+      </c>
+      <c r="C89" s="5">
+        <v>30</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="E89" s="28"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B90" s="38"/>
+      <c r="C90" s="8">
+        <v>10</v>
+      </c>
+      <c r="D90" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E90" s="28"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="7"/>
+      <c r="B91" s="38"/>
+      <c r="C91" s="8"/>
+      <c r="D91" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="E91" s="8"/>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="7"/>
+      <c r="B92" s="38"/>
+      <c r="C92" s="8"/>
+      <c r="D92" s="9"/>
+      <c r="E92" s="8"/>
+    </row>
+    <row r="93" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="10"/>
+      <c r="B93" s="39"/>
+      <c r="C93" s="10"/>
+      <c r="D93" s="11"/>
+      <c r="E93" s="10"/>
+    </row>
+    <row r="94" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B88" s="27"/>
-      <c r="C88" s="15">
-        <f>MROUND(SUM(C6:C60) /60,0.2)</f>
-        <v>25</v>
-      </c>
-      <c r="D88" s="16"/>
-      <c r="E88" s="17"/>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="18" t="s">
+      <c r="B94" s="27"/>
+      <c r="C94" s="15">
+        <f>MROUND(SUM(C6:C93) /60,0.2)</f>
+        <v>31</v>
+      </c>
+      <c r="D94" s="16"/>
+      <c r="E94" s="17"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="18" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2192,20 +2276,9 @@
       <c r="E153" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="B80:B87"/>
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B74:B78"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B46:B54"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B55:E55"/>
+  <mergeCells count="31">
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B89:B93"/>
     <mergeCell ref="B56:B60"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -2222,12 +2295,25 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B28:B32"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B46:B54"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B80:B87"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B74:B78"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78 C80:C87" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C56:C60 C143:C147 C40:C44 C16:C20 B6 C22:C26 C28:C32 C10:C14 C149:C153 C6:C8 C34:C38 C46:C54 C62:C66 C68:C72 C74:C78 C80:C87 C89:C93" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56 B62 B68 B74 B80" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B149:B153 B16:B20 B22:B26 B10:B14 B34:B38 B40:B44 B143:B147 B46 B28:B32 B56 B62 B68 B74 B80 B89" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2238,7 +2324,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="42" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="40" orientation="portrait" r:id="rId4"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2430,20 +2516,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="0dcbab57-ce0d-48ec-9006-afbf43b82b42" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2465,6 +2551,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -2478,12 +2572,4 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>